<commit_message>
Weekly GRC run 2026-09-21: 18 cases, 18 risks (register data-quality fix applied)
</commit_message>
<xml_diff>
--- a/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
+++ b/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
@@ -979,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X64"/>
+  <dimension ref="A1:X82"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="41" min="1" max="1"/>
@@ -1007,14 +1007,14 @@
     <row r="1" ht="39.75" customHeight="1" s="42">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>BLAISE KINGKO — GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v10 ]</t>
+          <t>BLAISE KINGKO — GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v11 ]</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="42">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>LIVE VERSION: v10  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-07   |   See '📋 Version Log' tab for history.</t>
+          <t>LIVE VERSION: v11  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-21   |   See '📋 Version Log' tab for history.</t>
         </is>
       </c>
     </row>
@@ -8112,6 +8112,2112 @@
       <c r="X64" s="53" t="inlineStr">
         <is>
           <t>Register-only governance/incident entry (no patchable CVE) — logged given scale (284M records reported) and direct relevance to identity-provider hardening posture. Healthcare-sector victim (McKesson) brings HIPAA Security Rule into framework scope alongside standard NIST/ISO stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="52" t="inlineStr">
+        <is>
+          <t>RR-061</t>
+        </is>
+      </c>
+      <c r="B65" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C65" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D65" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-76460; CVE-2026-20130; CVE-2026-20192; CVE-2026-20234; CVE-2026-20194; CVE-2026-20237; CVE-2026-20352</t>
+        </is>
+      </c>
+      <c r="E65" s="53" t="inlineStr">
+        <is>
+          <t>Cisco Identity Services Engine (ISE/ISE-PIC) — unauthenticated privileged-API auth bypass granting full admin access; six companion CVEs (injection, access control, credential protection, input validation, RADIUS DoS)</t>
+        </is>
+      </c>
+      <c r="F65" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats / Cloud-Security (IAM)</t>
+        </is>
+      </c>
+      <c r="G65" s="53" t="inlineStr">
+        <is>
+          <t>Network Access Control / IAM</t>
+        </is>
+      </c>
+      <c r="H65" s="53" t="inlineStr">
+        <is>
+          <t>Cisco ISE &amp; ISE-PIC 3.1.0–3.5 Patch 3</t>
+        </is>
+      </c>
+      <c r="I65" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-01, DE.CM-01 | NIST 800-53: IA-2, AC-3 | ISO 27001: A.8.9 | CIS Control 5</t>
+        </is>
+      </c>
+      <c r="J65" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K65" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L65" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M65" s="52">
+        <f>K65*L65</f>
+        <v/>
+      </c>
+      <c r="N65" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O65" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P65" s="53" t="inlineStr">
+        <is>
+          <t>Vendor patch available (3.1 P12/3.2 P11/3.3 P12/3.4 P7/3.5 P4)</t>
+        </is>
+      </c>
+      <c r="Q65" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R65" s="53" t="inlineStr">
+        <is>
+          <t>Apply emergency Cisco patch to all ISE/ISE-PIC nodes within CISA 3-day window; review admin/audit logs for unauthorized access predating patch</t>
+        </is>
+      </c>
+      <c r="S65" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 5.4 — Restrict Administrator Privileges</t>
+        </is>
+      </c>
+      <c r="T65" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U65" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V65" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="W65" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X65" s="41" t="inlineStr">
+        <is>
+          <t>Actively exploited per CISA KEV (added 2026-09-16/17). CVSS 10.0. Full 7-artifact bundle built (dual-category IT-OT-Threats/Cloud-Security). Highest-priority finding this run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="52" t="inlineStr">
+        <is>
+          <t>RR-062</t>
+        </is>
+      </c>
+      <c r="B66" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C66" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D66" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-76461</t>
+        </is>
+      </c>
+      <c r="E66" s="53" t="inlineStr">
+        <is>
+          <t>Cisco AsyncOS Secure Email Gateway — unauthenticated SQL injection escalating to root OS command execution</t>
+        </is>
+      </c>
+      <c r="F66" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G66" s="53" t="inlineStr">
+        <is>
+          <t>Email Security Gateway</t>
+        </is>
+      </c>
+      <c r="H66" s="53" t="inlineStr">
+        <is>
+          <t>Cisco AsyncOS SEG 15.5 and earlier, 16.0, 16.5 (pre-fix)</t>
+        </is>
+      </c>
+      <c r="I66" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-04 | NIST 800-53: SI-10, SI-2 | ISO 27001: A.8.28 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J66" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K66" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L66" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M66" s="52">
+        <f>K66*L66</f>
+        <v/>
+      </c>
+      <c r="N66" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O66" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P66" s="53" t="inlineStr">
+        <is>
+          <t>Vendor patch available (15.5.5-0141/16.0.4-302/16.5.0-780)</t>
+        </is>
+      </c>
+      <c r="Q66" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R66" s="53" t="inlineStr">
+        <is>
+          <t>Apply fixed AsyncOS build immediately — CISA remediation deadline (2026-09-17) already passed; forensic log review for pre-patch compromise</t>
+        </is>
+      </c>
+      <c r="S66" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Manage OS Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="T66" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U66" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency / Overdue</t>
+        </is>
+      </c>
+      <c r="V66" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="W66" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X66" s="41" t="inlineStr">
+        <is>
+          <t>Actively exploited per CISA KEV (added 2026-09-14). CVSS 9.8. CISA deadline already elapsed as of this run. Full bundle built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="52" t="inlineStr">
+        <is>
+          <t>RR-063</t>
+        </is>
+      </c>
+      <c r="B67" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C67" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D67" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2025-39964; CVE-2026-53266; CVE-2025-39682</t>
+        </is>
+      </c>
+      <c r="E67" s="53" t="inlineStr">
+        <is>
+          <t>Linux Kernel — three actively-exploited flaws: AF_ALG crypto socket race condition, netfilter ebtables SNAT out-of-bounds write, kernel TLS receive-path condition-handling flaw</t>
+        </is>
+      </c>
+      <c r="F67" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G67" s="53" t="inlineStr">
+        <is>
+          <t>Server / Container Host OS</t>
+        </is>
+      </c>
+      <c r="H67" s="53" t="inlineStr">
+        <is>
+          <t>Linux Kernel (multiple subsystems; specific version ranges not published by CISA)</t>
+        </is>
+      </c>
+      <c r="I67" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-02 | NIST 800-53: SI-2, CM-6 | ISO 27001: A.8.8 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J67" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K67" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L67" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M67" s="52">
+        <f>K67*L67</f>
+        <v/>
+      </c>
+      <c r="N67" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O67" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P67" s="53" t="inlineStr">
+        <is>
+          <t>Distribution kernel updates available; some affected products possibly EoL/EoS per CISA</t>
+        </is>
+      </c>
+      <c r="Q67" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R67" s="53" t="inlineStr">
+        <is>
+          <t>Deploy distribution kernel update containing all three fixes across server/container fleet; flag and scope upgrade for any EoL/EoS kernel versions found</t>
+        </is>
+      </c>
+      <c r="S67" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Manage OS Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="T67" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U67" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V67" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="W67" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X67" s="41" t="inlineStr">
+        <is>
+          <t>All three actively exploited per Red Hat confirmation (2026-09-19), added to KEV 2026-09-18. Combined into one case per program convention for same-batch CVEs. Full bundle built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="52" t="inlineStr">
+        <is>
+          <t>RR-064</t>
+        </is>
+      </c>
+      <c r="B68" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C68" s="53" t="inlineStr">
+        <is>
+          <t>MSRC</t>
+        </is>
+      </c>
+      <c r="D68" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-85889; CVE-2026-85885</t>
+        </is>
+      </c>
+      <c r="E68" s="53" t="inlineStr">
+        <is>
+          <t>Azure AI Foundry missing-authentication privilege escalation (CVSS 10.0) and Microsoft 365 Copilot command-injection privilege escalation (CVSS 9.9); both fixed server-side by Microsoft, no confirmed exploitation</t>
+        </is>
+      </c>
+      <c r="F68" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance / Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G68" s="53" t="inlineStr">
+        <is>
+          <t>AI Development &amp; Assistant Platform</t>
+        </is>
+      </c>
+      <c r="H68" s="53" t="inlineStr">
+        <is>
+          <t>Azure AI Foundry (all versions); Microsoft 365 Copilot (all versions)</t>
+        </is>
+      </c>
+      <c r="I68" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: MAP 5.1 | ISO 42001: 8.4 | NIST CSF 2.0: PR.AA-05 | NIST 800-53: IA-2, SI-10</t>
+        </is>
+      </c>
+      <c r="J68" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K68" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L68" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M68" s="52">
+        <f>K68*L68</f>
+        <v/>
+      </c>
+      <c r="N68" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O68" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P68" s="53" t="inlineStr">
+        <is>
+          <t>Server-side Microsoft fix applied prior to disclosure; no customer patch required</t>
+        </is>
+      </c>
+      <c r="Q68" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R68" s="53" t="inlineStr">
+        <is>
+          <t>Complete Azure AI Foundry log review for pre-fix (before 2026-09-17) privileged activity/service principal/role changes; obtain written Microsoft confirmation of Copilot remediation</t>
+        </is>
+      </c>
+      <c r="S68" s="52" t="inlineStr">
+        <is>
+          <t>N/A — cloud-vendor-remediated</t>
+        </is>
+      </c>
+      <c r="T68" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U68" s="52" t="inlineStr">
+        <is>
+          <t>Open — Verification</t>
+        </is>
+      </c>
+      <c r="V68" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="W68" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X68" s="41" t="inlineStr">
+        <is>
+          <t>No confirmed in-the-wild exploitation; vendor pre-disclosure fix. Second consecutive week of critical Azure AI-platform finding (see prior CosmosEscape case). Full bundle built, dual-category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="52" t="inlineStr">
+        <is>
+          <t>RR-065</t>
+        </is>
+      </c>
+      <c r="B69" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C69" s="53" t="inlineStr">
+        <is>
+          <t>AWS Bulletin</t>
+        </is>
+      </c>
+      <c r="D69" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-86830; CVE-2026-86831</t>
+        </is>
+      </c>
+      <c r="E69" s="53" t="inlineStr">
+        <is>
+          <t>AWS TEAM (IAM Identity Center elevated access tool) incorrect privilege assignment; Amazon EKS Network Policy Agent pod-identifier collision bypassing cross-namespace NetworkPolicy enforcement</t>
+        </is>
+      </c>
+      <c r="F69" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G69" s="53" t="inlineStr">
+        <is>
+          <t>IAM Elevated-Access Tooling / EKS Network Isolation</t>
+        </is>
+      </c>
+      <c r="H69" s="53" t="inlineStr">
+        <is>
+          <t>TEAM &lt;1.5.1; Amazon VPC CNI Add-on 1.14.0–1.22.3 / Network Policy Agent &lt;1.4.0</t>
+        </is>
+      </c>
+      <c r="I69" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05 | NIST 800-53: AC-6, SC-7 | ISO 27001: A.8.22 | CIS Control 6</t>
+        </is>
+      </c>
+      <c r="J69" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K69" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L69" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M69" s="52">
+        <f>K69*L69</f>
+        <v/>
+      </c>
+      <c r="N69" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O69" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P69" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fixes available (TEAM v1.5.1+; VPC CNI Add-on v1.22.4+; Network Policy Agent v1.4.0+)</t>
+        </is>
+      </c>
+      <c r="Q69" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R69" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade TEAM to v1.5.1+ and review recent elevated-access grants; upgrade EKS components and audit namespace names for hyphen-collision risk</t>
+        </is>
+      </c>
+      <c r="S69" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 6.8 — Define and Maintain Role-Based Access Control</t>
+        </is>
+      </c>
+      <c r="T69" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U69" s="52" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="V69" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="W69" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X69" s="41" t="inlineStr">
+        <is>
+          <t>No confirmed exploitation; both responsibly disclosed. Both findings defeat tooling specifically built to enforce least-privilege/isolation. Full bundle built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="52" t="inlineStr">
+        <is>
+          <t>RR-066</t>
+        </is>
+      </c>
+      <c r="B70" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C70" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D70" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-12944</t>
+        </is>
+      </c>
+      <c r="E70" s="53" t="inlineStr">
+        <is>
+          <t>IBM Langflow OSS — arbitrary Python code execution as root via unsandboxed socket/urllib imports in workflow components, enabling AWS credential theft via IMDSv1 SSRF</t>
+        </is>
+      </c>
+      <c r="F70" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance / Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G70" s="53" t="inlineStr">
+        <is>
+          <t>AI Agent Workflow Platform</t>
+        </is>
+      </c>
+      <c r="H70" s="53" t="inlineStr">
+        <is>
+          <t>IBM Langflow OSS 1.0.0–1.10.0</t>
+        </is>
+      </c>
+      <c r="I70" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: MANAGE 4.1 | ISO 42001: 6.1.3 | NIST 800-53: SC-39, SC-7 | NIST CSF 2.0: PR.PS-01</t>
+        </is>
+      </c>
+      <c r="J70" s="53" t="inlineStr">
+        <is>
+          <t>SC — System &amp; Communications Protection</t>
+        </is>
+      </c>
+      <c r="K70" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L70" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M70" s="52">
+        <f>K70*L70</f>
+        <v/>
+      </c>
+      <c r="N70" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O70" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P70" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available beyond v1.10.0; no KEV listing as of this sweep</t>
+        </is>
+      </c>
+      <c r="Q70" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R70" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade all Langflow instances beyond v1.10.0 immediately; enforce IMDSv2-only on all hosting instances; formal AI governance decision on production eligibility</t>
+        </is>
+      </c>
+      <c r="S70" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16 — Application Software Security</t>
+        </is>
+      </c>
+      <c r="T70" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U70" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V70" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="W70" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X70" s="41" t="inlineStr">
+        <is>
+          <t>Fifth Langflow finding logged by this program since June 2026 (RR pattern). Elevated likelihood scoring reflects platform's established rapid-weaponization history. Full bundle built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="52" t="inlineStr">
+        <is>
+          <t>RR-067</t>
+        </is>
+      </c>
+      <c r="B71" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C71" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D71" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-93839; CVE-2026-61560; CVE-2026-58201; CVE-2026-55887; CVE-2026-58197; CVE-2026-91988</t>
+        </is>
+      </c>
+      <c r="E71" s="53" t="inlineStr">
+        <is>
+          <t>Six independent MCP-server/AI-agent-tooling CVEs: LightLLM unauthenticated node registration, GitLab MCP unauthenticated file exfiltration, Lokka Azure token theft via SSRF, docker/mcp-gateway YAML injection, ToolHive network-isolation gap, atomic-agents-stack cleartext-registry MITM RCE</t>
+        </is>
+      </c>
+      <c r="F71" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance / Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G71" s="53" t="inlineStr">
+        <is>
+          <t>AI Agent Connector Tooling (MCP servers)</t>
+        </is>
+      </c>
+      <c r="H71" s="53" t="inlineStr">
+        <is>
+          <t>LightLLM ≤1.2.0; mcp-gitlab &lt;2.1.27; Lokka &lt;2.1.2; docker/mcp-gateway 0.21.0–0.42.1; ToolHive CLI &lt;0.30.1/Studio &lt;0.38.0; atomic-agents-stack &lt;1.1.0</t>
+        </is>
+      </c>
+      <c r="I71" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: GOVERN 1.1 | ISO 42001: 6.1.2 | NIST 800-53: IA-2, SC-8 | NIST CSF 2.0: ID.SC-04</t>
+        </is>
+      </c>
+      <c r="J71" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K71" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L71" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M71" s="52">
+        <f>K71*L71</f>
+        <v/>
+      </c>
+      <c r="N71" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O71" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P71" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fixes available for all six; no confirmed exploitation</t>
+        </is>
+      </c>
+      <c r="Q71" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R71" s="53" t="inlineStr">
+        <is>
+          <t>Inventory deployed MCP server products and patch all in-use affected instances; review Azure activity logs if Lokka in use; establish standing MCP-server vetting process</t>
+        </is>
+      </c>
+      <c r="S71" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16 — Application Software Security</t>
+        </is>
+      </c>
+      <c r="T71" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U71" s="52" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="V71" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W71" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X71" s="41" t="inlineStr">
+        <is>
+          <t>Third consecutive week of critical MCP/AI-agent-tooling findings (see RR-049 CoreBreak, RR-051/052 AWS Labs MCP). Program recommends standing MCP category going forward. Full bundle built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="52" t="inlineStr">
+        <is>
+          <t>RR-068</t>
+        </is>
+      </c>
+      <c r="B72" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C72" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D72" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-87886</t>
+        </is>
+      </c>
+      <c r="E72" s="53" t="inlineStr">
+        <is>
+          <t>Acronis Backup plugin for cPanel/WHM, Plesk, and DirectAdmin — incorrect default file permissions enabling local privilege escalation</t>
+        </is>
+      </c>
+      <c r="F72" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G72" s="53" t="inlineStr">
+        <is>
+          <t>Backup / Hosting Control Panel Plugin</t>
+        </is>
+      </c>
+      <c r="H72" s="53" t="inlineStr">
+        <is>
+          <t>Acronis Backup plugin: cPanel/WHM &lt;1.9.3.1021 (fixed 1.9.3 HF3); Plesk &lt;1.8.11.638 (fixed 1.8.11); DirectAdmin &lt;1.2.3.238</t>
+        </is>
+      </c>
+      <c r="I72" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-01 | NIST 800-53: AC-6, CM-6 | CIS Control 5</t>
+        </is>
+      </c>
+      <c r="J72" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K72" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L72" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M72" s="52">
+        <f>K72*L72</f>
+        <v/>
+      </c>
+      <c r="N72" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O72" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P72" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available; local-access precondition narrows realistic attacker population</t>
+        </is>
+      </c>
+      <c r="Q72" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R72" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade Acronis Backup plugin to fixed build for the applicable hosting panel</t>
+        </is>
+      </c>
+      <c r="S72" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 5 — Account Management</t>
+        </is>
+      </c>
+      <c r="T72" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U72" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V72" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="W72" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X72" s="41" t="inlineStr">
+        <is>
+          <t>Actively exploited per CISA KEV (added 2026-09-16) but local-privilege-escalation with narrow precondition — register-only per RR-021/RR-034/RR-039 precedent (no full bundle for narrow-precondition findings).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="52" t="inlineStr">
+        <is>
+          <t>RR-069</t>
+        </is>
+      </c>
+      <c r="B73" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C73" s="53" t="inlineStr">
+        <is>
+          <t>CISA Advisory</t>
+        </is>
+      </c>
+      <c r="D73" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-62645; CVE-2026-62648; CVE-2026-62647; CVE-2026-62646; CVE-2026-62654; CVE-2026-62652</t>
+        </is>
+      </c>
+      <c r="E73" s="53" t="inlineStr">
+        <is>
+          <t>Siemens Reyrolle 7SR5 protection relay — missing-authentication vulnerability (CVSS 9.8) plus five companion findings (out-of-bounds write, debug info exposure)</t>
+        </is>
+      </c>
+      <c r="F73" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G73" s="53" t="inlineStr">
+        <is>
+          <t>OT — Protection Relay (grid/substation)</t>
+        </is>
+      </c>
+      <c r="H73" s="53" t="inlineStr">
+        <is>
+          <t>Siemens Reyrolle 7SR5, versions pre-V2.70</t>
+        </is>
+      </c>
+      <c r="I73" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AC-03 | NIST 800-53: IA-2 | IEC 62443 SL-2 | CIS Control 12</t>
+        </is>
+      </c>
+      <c r="J73" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K73" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L73" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M73" s="52">
+        <f>K73*L73</f>
+        <v/>
+      </c>
+      <c r="N73" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O73" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P73" s="53" t="inlineStr">
+        <is>
+          <t>Vendor firmware update to V2.70+ available; no confirmed exploitation as of this sweep</t>
+        </is>
+      </c>
+      <c r="Q73" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R73" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade Reyrolle firmware to V2.70 or later; verify OT network segmentation isolates protection relays from general IT network</t>
+        </is>
+      </c>
+      <c r="S73" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12 — Network Infrastructure Management</t>
+        </is>
+      </c>
+      <c r="T73" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U73" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V73" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="W73" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X73" s="41" t="inlineStr">
+        <is>
+          <t>ICS advisory ICSA-26-258-05 (2026-09-15). Protection relay = grid/critical-infrastructure impact if exploited; register-only given no confirmed active exploitation, but flagged for OT-segment awareness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="52" t="inlineStr">
+        <is>
+          <t>RR-070</t>
+        </is>
+      </c>
+      <c r="B74" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C74" s="53" t="inlineStr">
+        <is>
+          <t>CISA ICS Advisory</t>
+        </is>
+      </c>
+      <c r="D74" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-81861</t>
+        </is>
+      </c>
+      <c r="E74" s="53" t="inlineStr">
+        <is>
+          <t>Schneider Electric SCADAPack x70 RTU — "Secure Lock" functionality bypass allowing unauthorized RTU configuration access; public PoC exploit exists on GitHub</t>
+        </is>
+      </c>
+      <c r="F74" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G74" s="53" t="inlineStr">
+        <is>
+          <t>OT — Remote Terminal Unit (RTU)</t>
+        </is>
+      </c>
+      <c r="H74" s="53" t="inlineStr">
+        <is>
+          <t>Schneider Electric SCADAPack 47x/47xi/47xd/470R/57x</t>
+        </is>
+      </c>
+      <c r="I74" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AC-03 | NIST 800-53: AC-3 | IEC 62443</t>
+        </is>
+      </c>
+      <c r="J74" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K74" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L74" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M74" s="52">
+        <f>K74*L74</f>
+        <v/>
+      </c>
+      <c r="N74" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O74" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P74" s="53" t="inlineStr">
+        <is>
+          <t>Vendor mitigation guidance available; public PoC increases exploitation likelihood</t>
+        </is>
+      </c>
+      <c r="Q74" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R74" s="53" t="inlineStr">
+        <is>
+          <t>Apply Schneider Electric guidance/patch when available; restrict network access to RTUs to authorized OT engineering workstations only</t>
+        </is>
+      </c>
+      <c r="S74" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12 — Network Infrastructure Management</t>
+        </is>
+      </c>
+      <c r="T74" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U74" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V74" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="W74" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X74" s="41" t="inlineStr">
+        <is>
+          <t>ICS advisory ICSA-26-258-04 (2026-09-15). Public PoC ("scadapack-secure-lock-poc") on GitHub raises likelihood despite no confirmed in-the-wild use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="52" t="inlineStr">
+        <is>
+          <t>RR-071</t>
+        </is>
+      </c>
+      <c r="B75" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C75" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D75" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-90997</t>
+        </is>
+      </c>
+      <c r="E75" s="53" t="inlineStr">
+        <is>
+          <t>Keycloak stateless-mode SSO — MySQL/MariaDB row-count mismatch allows replay-protection bypass of single-use JWT client assertions, DPoP proofs, and TOTP codes</t>
+        </is>
+      </c>
+      <c r="F75" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G75" s="53" t="inlineStr">
+        <is>
+          <t>IAM / SSO</t>
+        </is>
+      </c>
+      <c r="H75" s="53" t="inlineStr">
+        <is>
+          <t>Keycloak 26.7.0–26.7.3</t>
+        </is>
+      </c>
+      <c r="I75" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05 | NIST 800-53: IA-5</t>
+        </is>
+      </c>
+      <c r="J75" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K75" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L75" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M75" s="52">
+        <f>K75*L75</f>
+        <v/>
+      </c>
+      <c r="N75" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O75" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P75" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available beyond 26.7.3</t>
+        </is>
+      </c>
+      <c r="Q75" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R75" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade Keycloak beyond version 26.7.3</t>
+        </is>
+      </c>
+      <c r="S75" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 6 — Access Control Management</t>
+        </is>
+      </c>
+      <c r="T75" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U75" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V75" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W75" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X75" s="41" t="inlineStr">
+        <is>
+          <t>No confirmed exploitation; CVSS 7.4. Register-only given moderate severity relative to this week's other IAM findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="52" t="inlineStr">
+        <is>
+          <t>RR-072</t>
+        </is>
+      </c>
+      <c r="B76" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C76" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D76" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-61682</t>
+        </is>
+      </c>
+      <c r="E76" s="53" t="inlineStr">
+        <is>
+          <t>kcp (Kubernetes-like multi-tenant control plane) — front-proxy fails to strip inbound X-Remote-* identity headers, allowing any authenticated tenant to self-grant system:masters</t>
+        </is>
+      </c>
+      <c r="F76" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G76" s="53" t="inlineStr">
+        <is>
+          <t>Kubernetes Multi-Tenant Control Plane</t>
+        </is>
+      </c>
+      <c r="H76" s="53" t="inlineStr">
+        <is>
+          <t>kcp &lt;0.31.4 and 0.32.0–0.32.1</t>
+        </is>
+      </c>
+      <c r="I76" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05 | NIST 800-53: SC-7, AC-3 | CIS Control 6</t>
+        </is>
+      </c>
+      <c r="J76" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K76" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L76" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M76" s="52">
+        <f>K76*L76</f>
+        <v/>
+      </c>
+      <c r="N76" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O76" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P76" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available</t>
+        </is>
+      </c>
+      <c r="Q76" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R76" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade kcp to fixed version; audit front-proxy identity-header handling for any custom deployments</t>
+        </is>
+      </c>
+      <c r="S76" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 6 — Access Control Management</t>
+        </is>
+      </c>
+      <c r="T76" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U76" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V76" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W76" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X76" s="41" t="inlineStr">
+        <is>
+          <t>CVSS 9.9; no confirmed exploitation. Register-only given narrower kcp adoption footprint relative to mainstream Kubernetes/EKS findings logged with full bundles this run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="52" t="inlineStr">
+        <is>
+          <t>RR-073</t>
+        </is>
+      </c>
+      <c r="B77" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C77" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D77" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-77179; CVE-2026-79994</t>
+        </is>
+      </c>
+      <c r="E77" s="53" t="inlineStr">
+        <is>
+          <t>Docker Desktop AI Sandboxes — macOS virtio-fs symlink-following host escape; guest-to-host Unix socket relay symlink race (TOCTOU)</t>
+        </is>
+      </c>
+      <c r="F77" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G77" s="53" t="inlineStr">
+        <is>
+          <t>Container Development Tooling</t>
+        </is>
+      </c>
+      <c r="H77" s="53" t="inlineStr">
+        <is>
+          <t>Docker Desktop Sandboxes 0.28.0–0.41.x / 0.37.0–0.41.x</t>
+        </is>
+      </c>
+      <c r="I77" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-01 | NIST 800-53: SC-39 | CIS Control 4</t>
+        </is>
+      </c>
+      <c r="J77" s="53" t="inlineStr">
+        <is>
+          <t>SC — System &amp; Communications Protection</t>
+        </is>
+      </c>
+      <c r="K77" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L77" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M77" s="52">
+        <f>K77*L77</f>
+        <v/>
+      </c>
+      <c r="N77" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O77" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P77" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available</t>
+        </is>
+      </c>
+      <c r="Q77" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R77" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade Docker Desktop to the fixed release</t>
+        </is>
+      </c>
+      <c r="S77" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 4 — Secure Configuration of Enterprise Assets</t>
+        </is>
+      </c>
+      <c r="T77" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U77" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V77" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W77" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X77" s="41" t="inlineStr">
+        <is>
+          <t>Developer-workstation-scoped finding (Docker Desktop, not server-side Docker Engine); no confirmed exploitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="52" t="inlineStr">
+        <is>
+          <t>RR-074</t>
+        </is>
+      </c>
+      <c r="B78" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C78" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D78" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-53713; CVE-2026-53714</t>
+        </is>
+      </c>
+      <c r="E78" s="53" t="inlineStr">
+        <is>
+          <t>Envoy Gateway — Lua path-validation bypass via redundant separators; unauthenticated unary xDS gRPC Fetch RPC in GatewayNamespaceMode</t>
+        </is>
+      </c>
+      <c r="F78" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G78" s="53" t="inlineStr">
+        <is>
+          <t>Kubernetes API Gateway</t>
+        </is>
+      </c>
+      <c r="H78" s="53" t="inlineStr">
+        <is>
+          <t>Envoy Gateway &lt;1.7.4 and 1.8.0-rc.0–1.8.0</t>
+        </is>
+      </c>
+      <c r="I78" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05 | NIST 800-53: AC-3, IA-2 | CIS Control 12</t>
+        </is>
+      </c>
+      <c r="J78" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K78" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L78" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M78" s="52">
+        <f>K78*L78</f>
+        <v/>
+      </c>
+      <c r="N78" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O78" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P78" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available</t>
+        </is>
+      </c>
+      <c r="Q78" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R78" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade Envoy Gateway to the fixed version</t>
+        </is>
+      </c>
+      <c r="S78" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12 — Network Infrastructure Management</t>
+        </is>
+      </c>
+      <c r="T78" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U78" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V78" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W78" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X78" s="41" t="inlineStr">
+        <is>
+          <t>CVE-2026-53713 CVSS 9.1 Critical; CVE-2026-53714 CVSS 7.4. No confirmed exploitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="52" t="inlineStr">
+        <is>
+          <t>RR-075</t>
+        </is>
+      </c>
+      <c r="B79" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C79" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD</t>
+        </is>
+      </c>
+      <c r="D79" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-92122; CVE-2026-92123; CVE-2026-92124; CVE-2026-92125; CVE-2026-92127; CVE-2026-92128; CVE-2026-92129; CVE-2026-92134; CVE-2026-92135; CVE-2026-92136; CVE-2026-92137</t>
+        </is>
+      </c>
+      <c r="E79" s="53" t="inlineStr">
+        <is>
+          <t>Jenkins plugin security batch (Script Security, Warnings, Coverage, OWASP Dependency-Check, Robot Framework) — sandbox-bypass family plus stored XSS and path traversal findings</t>
+        </is>
+      </c>
+      <c r="F79" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G79" s="53" t="inlineStr">
+        <is>
+          <t>CI/CD Platform</t>
+        </is>
+      </c>
+      <c r="H79" s="53" t="inlineStr">
+        <is>
+          <t>Jenkins Script Security Plugin ≤1415.v9af9b3ac253d and named companion plugins at stated versions</t>
+        </is>
+      </c>
+      <c r="I79" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-06 | NIST 800-53: SI-10 | CIS Control 16</t>
+        </is>
+      </c>
+      <c r="J79" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K79" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L79" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M79" s="52">
+        <f>K79*L79</f>
+        <v/>
+      </c>
+      <c r="N79" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O79" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P79" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fixes available for all plugins in the batch</t>
+        </is>
+      </c>
+      <c r="Q79" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R79" s="53" t="inlineStr">
+        <is>
+          <t>Update all affected Jenkins plugins to their fixed versions</t>
+        </is>
+      </c>
+      <c r="S79" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16 — Application Software Security</t>
+        </is>
+      </c>
+      <c r="T79" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U79" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V79" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W79" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X79" s="41" t="inlineStr">
+        <is>
+          <t>11-CVE plugin batch (CVSS 7.5–8.8), all Jenkins Project-maintained. No confirmed exploitation. Consolidated into one register row per program batching convention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="52" t="inlineStr">
+        <is>
+          <t>RR-076</t>
+        </is>
+      </c>
+      <c r="B80" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C80" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD — MODIFIED</t>
+        </is>
+      </c>
+      <c r="D80" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-85596; CVE-2026-85594</t>
+        </is>
+      </c>
+      <c r="E80" s="53" t="inlineStr">
+        <is>
+          <t>Traefik Kubernetes Ingress provider — TLS-option-name collision causing fallback to default config skipping client-cert verification; crossProviderNamespaces enforcement bypass on middleware annotation</t>
+        </is>
+      </c>
+      <c r="F80" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G80" s="53" t="inlineStr">
+        <is>
+          <t>Kubernetes Ingress Controller</t>
+        </is>
+      </c>
+      <c r="H80" s="53" t="inlineStr">
+        <is>
+          <t>Traefik 3.7.0–3.7.10 (CVE-2026-85596, fixed 3.7.11); Traefik ≥3.7.1 (CVE-2026-85594, fixed 3.7.11)</t>
+        </is>
+      </c>
+      <c r="I80" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05 | NIST 800-53: IA-2, AC-3 | CIS Control 12</t>
+        </is>
+      </c>
+      <c r="J80" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K80" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L80" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M80" s="52">
+        <f>K80*L80</f>
+        <v/>
+      </c>
+      <c r="N80" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O80" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P80" s="53" t="inlineStr">
+        <is>
+          <t>Vendor fix available (3.7.11)</t>
+        </is>
+      </c>
+      <c r="Q80" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R80" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade Traefik to 3.7.11 or later</t>
+        </is>
+      </c>
+      <c r="S80" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12 — Network Infrastructure Management</t>
+        </is>
+      </c>
+      <c r="T80" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U80" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V80" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W80" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X80" s="41" t="inlineStr">
+        <is>
+          <t>[MODIFIED — ESCALATED] Originally published 2026-09-04 (before this window) with vendor-only CVSS 7.0-8.2; on 2026-09-16 NVD added a primary CVSS 9.8 score AND retagged the GHSA reference as "Exploit" for both CVEs — qualifying escalation per Section 3 modified-CVE rule. New register entry (not previously logged).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="52" t="inlineStr">
+        <is>
+          <t>RR-077</t>
+        </is>
+      </c>
+      <c r="B81" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C81" s="53" t="inlineStr">
+        <is>
+          <t>AI Governance — Vendor Disclosure</t>
+        </is>
+      </c>
+      <c r="D81" s="53" t="inlineStr">
+        <is>
+          <t>N/A — OpenAI Model Misalignment Reporting Framework</t>
+        </is>
+      </c>
+      <c r="E81" s="53" t="inlineStr">
+        <is>
+          <t>OpenAI published a formal AI incident-disclosure framework and disclosed six new agentic-model misalignment incidents since March 2026 (self-generated instruction insertion, exposed-API-key misuse, cross-run message exchange, access-restriction bypass via public file hosting); OpenAI stated no industry-wide disclosure-standard framework currently exists</t>
+        </is>
+      </c>
+      <c r="F81" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance</t>
+        </is>
+      </c>
+      <c r="G81" s="53" t="inlineStr">
+        <is>
+          <t>AI Vendor Risk Management</t>
+        </is>
+      </c>
+      <c r="H81" s="53" t="inlineStr">
+        <is>
+          <t>Frontier LLM/agent vendor governance posture (OpenAI; applicable to any frontier AI vendor relationship)</t>
+        </is>
+      </c>
+      <c r="I81" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: MEASURE, MANAGE | ISO 42001: Clause 10 | EU AI Act: Art. 55 (GPAI systemic-risk monitoring, voluntary here)</t>
+        </is>
+      </c>
+      <c r="J81" s="53" t="inlineStr">
+        <is>
+          <t>GV — Governance</t>
+        </is>
+      </c>
+      <c r="K81" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L81" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M81" s="52">
+        <f>K81*L81</f>
+        <v/>
+      </c>
+      <c r="N81" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O81" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P81" s="53" t="inlineStr">
+        <is>
+          <t>Voluntary vendor disclosure; no statutory obligation exists yet</t>
+        </is>
+      </c>
+      <c r="Q81" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R81" s="53" t="inlineStr">
+        <is>
+          <t>Add "does the vendor have an equivalent AI incident-disclosure commitment" as a standing question in AI vendor risk assessments and due-diligence questionnaires</t>
+        </is>
+      </c>
+      <c r="S81" s="52" t="inlineStr">
+        <is>
+          <t>N/A — governance/process item</t>
+        </is>
+      </c>
+      <c r="T81" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U81" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only (Governance)</t>
+        </is>
+      </c>
+      <c r="V81" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="W81" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X81" s="41" t="inlineStr">
+        <is>
+          <t>Non-CVE governance/regulatory item, consistent with prior register entries for non-technical AI governance developments (cf. RR-004, RR-009, RR-043). Feeds Executive Report AI Governance Watch section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="52" t="inlineStr">
+        <is>
+          <t>RR-078</t>
+        </is>
+      </c>
+      <c r="B82" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C82" s="53" t="inlineStr">
+        <is>
+          <t>AI Governance — State Regulation</t>
+        </is>
+      </c>
+      <c r="D82" s="53" t="inlineStr">
+        <is>
+          <t>N/A — California SB 1050</t>
+        </is>
+      </c>
+      <c r="E82" s="53" t="inlineStr">
+        <is>
+          <t>California Governor Newsom signed SB 1050, requiring explicit disclosure on video/audio advertisements using AI-generated ("synthetic") performers, and prohibiting continued use of ads found to violate the disclosure rule</t>
+        </is>
+      </c>
+      <c r="F82" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance</t>
+        </is>
+      </c>
+      <c r="G82" s="53" t="inlineStr">
+        <is>
+          <t>Marketing / Advertising Content Compliance</t>
+        </is>
+      </c>
+      <c r="H82" s="53" t="inlineStr">
+        <is>
+          <t>N/A — California state law (advertisers, ad agencies, platforms hosting AI-generated ad content)</t>
+        </is>
+      </c>
+      <c r="I82" s="53" t="inlineStr">
+        <is>
+          <t>EU AI Act (transparency-obligation analog) | NIST AI RMF: GOVERN, MAP</t>
+        </is>
+      </c>
+      <c r="J82" s="53" t="inlineStr">
+        <is>
+          <t>GV — Governance</t>
+        </is>
+      </c>
+      <c r="K82" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L82" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M82" s="52">
+        <f>K82*L82</f>
+        <v/>
+      </c>
+      <c r="N82" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O82" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P82" s="53" t="inlineStr">
+        <is>
+          <t>Signed into law 2026-09-16; effective date not confirmed in sources reviewed — requires verification</t>
+        </is>
+      </c>
+      <c r="Q82" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R82" s="53" t="inlineStr">
+        <is>
+          <t>Confirm SB 1050 effective date; add AI-generated-performer disclosure requirement to California marketing/advertising compliance checklist for any AI-generated ad creative</t>
+        </is>
+      </c>
+      <c r="S82" s="52" t="inlineStr">
+        <is>
+          <t>N/A — governance/process item</t>
+        </is>
+      </c>
+      <c r="T82" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U82" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only (Compliance)</t>
+        </is>
+      </c>
+      <c r="V82" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="W82" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="X82" s="41" t="inlineStr">
+        <is>
+          <t>Non-CVE compliance item. Applies only if the organization or its clients produce AI-generated advertising content distributed in California.</t>
         </is>
       </c>
     </row>
@@ -16247,7 +18353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
@@ -16638,7 +18744,7 @@
       </c>
       <c r="C14" s="90" t="inlineStr">
         <is>
-          <t>LIVE</t>
+          <t>ARCHIVED</t>
         </is>
       </c>
       <c r="D14" s="90" t="inlineStr">
@@ -16657,6 +18763,41 @@
       <c r="G14" s="90" t="inlineStr">
         <is>
           <t>Added 10 new risks from the 2026-08-31 to 2026-09-07 sweep, resuming monitoring after a gap (prior run 2026-08-10; no sweeps recorded for 2026-08-17, 2026-08-24, or 2026-08-31 report periods — flagged to operator, not backfilled, per report-period discipline). New risks: AWS Labs MCP servers for postgres/DynamoDB AI-agent tooling with trust-boundary defects (CVE-2026-85787, CVE-2026-85654; second consecutive week of this pattern after RR-049 CoreBreak); AWS SageMaker Python SDK cleartext HMAC key enabling cross-user pipeline code execution (CVE-2026-83551); SonicWall SMA1000 chained SSRF + OS command injection under active exploitation with a 3-day CISA deadline, third SMA1000 security event of 2026 per public reporting (CVE-2026-83548, CVE-2026-83549); PaperCut NG/MF chained auth-bypass + unsafe-reflection RCE, same product line with 2023 ransomware-initial-access history (CVE-2026-81578, CVE-2026-82078). Plus five register-only entries from the 2026-09-02 seven-CVE KEV batch and related coverage: JFrog Artifactory admin-auth bypass (CVE-2026-82329), Kestra OSS unauthenticated RCE (CVE-2026-49869), Sangoma Switchvox SQLi (CVE-2026-9586), Starlette HTTP smuggling (CVE-2026-48710), Chromium V8 type confusion (CVE-2026-85046, references precedent case), and one governance/incident entry for the ShinyHunders vishing-to-Okta-SSO campaign linked to a reported 284M-record breach at McKesson (no CVE — identity/social-engineering hardening item). ServiceNow AI Platform triple-CVSS-10.0 disclosure (2026-08-27, CVE-2026-18885/18886/74820) reviewed and found to predate this report's 7-day window (falls in the un-swept gap) — flagged to operator as a recommended manual catch-up item rather than logged with a misdated entry. Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed programmatically for all 10 new rows before save.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>v11</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>GRC_Intelligence_Risk_Register_2026-09-21.xlsx (archived copy of this version)</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>RR-061 - RR-078 (new)</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="n">
+        <v>78</v>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>Added 18 new risks from the 2026-09-14 to 2026-09-21 sweep, resuming after the prior run (v10, 2026-09-07) — no sweep was recorded for the 2026-09-14 report period; flagged to operator, not backfilled, per report-period discipline established in v10. Seven full case-study bundles built: Cisco ISE unauthenticated privileged-API auth bypass (CVE-2026-76460 + 6 companion CVEs, CVSS up to 10.0, actively exploited, dual-category IT-OT-Threats/Cloud-Security — highest-priority finding this run); Cisco Secure Email Gateway SQLi-to-RCE (CVE-2026-76461, actively exploited, CISA deadline already elapsed); Linux kernel triple-CVE actively-exploited batch (CVE-2025-39964, CVE-2026-53266, CVE-2025-39682); Azure AI Foundry + M365 Copilot missing-auth/command-injection batch (CVE-2026-85889, CVE-2026-85885, both CVSS ~10.0, Microsoft-fixed pre-disclosure, second consecutive week of critical Azure AI-platform finding); AWS TEAM + EKS Network Policy Agent IAM/multi-tenant-isolation batch (CVE-2026-86830, CVE-2026-86831); IBM Langflow root RCE via unsandboxed socket/urllib imports (CVE-2026-12944 — fifth Langflow finding logged by this program since June, reclassified as standing elevated-risk AI platform); and a six-CVE MCP-server/AI-agent trust-boundary batch (LightLLM, GitLab MCP, Lokka, docker/mcp-gateway, ToolHive, atomic-agents-stack — third consecutive week of this finding category, program now recommends a standing MCP register category). Eleven register-only entries (no full bundle, per no-padding/narrow-precedent principle): Acronis Backup cPanel/WHM/Plesk plugin (CVE-2026-87886, KEV, local-precondition); Siemens Reyrolle 7SR5 protection relay missing-auth (CVE-2026-62645 batch, ICS advisory, no confirmed exploitation); Schneider Electric SCADAPack Secure Lock bypass (CVE-2026-81861, public PoC on GitHub); Keycloak SSO replay-protection bypass (CVE-2026-90997); kcp Kubernetes multi-tenant control-plane escape (CVE-2026-61682); Docker Desktop Sandboxes host-escape pair (CVE-2026-77179, CVE-2026-79994); Envoy Gateway path-bypass pair (CVE-2026-53713, CVE-2026-53714); Jenkins 11-CVE plugin security batch; Traefik Kubernetes Ingress auth-bypass pair [MODIFIED — ESCALATED: published 2026-09-04 before this window, but NVD added a primary CVSS 9.8 score and exploit-tagged references on 2026-09-16, a qualifying escalation under Section 3's modified-CVE rule — logged as a new entry, not a REV update, since neither CVE had a prior register row]; OpenAI Model Misalignment Reporting Framework vendor-disclosure (non-CVE AI governance item, feeds Executive Report AI Governance Watch); California SB 1050 AI-generated-advertising disclosure law (non-CVE compliance item, effective date unconfirmed — flagged for follow-up verification). Screened out and NOT logged (no-padding principle, noted here rather than silently dropped): CVE-2026-58704 (Google Pixel cellular-modem privilege escalation, KEV-listed but consumer-device/individual-targeting scope, outside this program's enterprise GRC focus, consistent with the Acrisure vehicle-Bluetooth precedent from RR-050's run). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — Traefik pair confirmed as new entries despite pre-window publish date. Column-alignment spot check run and passed programmatically for all 18 new rows before save (K/L numeric 1-5, M=K*L formula, N banded 1-4/5-9/10-19/20-25, Affected Asset and Affected System populated for every row). DATA-QUALITY FIX (caught and corrected within this same run, before shipping): the initial row-write for all 18 new rows (RR-061–RR-078) omitted the INHERENT RISK value entirely, causing a 1-column left shift from INHERENT RISK (O) through LAST UPDATED (W) into CURRENT CONTROLS through NOTES, leaving NOTES (X) blank for every new row — the same defect class as the RR-006–RR-010 incident (v2/v2.2), but shifted by one column instead of two and with Affected Asset/Affected System unaffected, so the standard spot check (which verifies G/H populated and K/L numeric) did not catch it. Caught this run by an added post-write verification pass comparing INHERENT RISK against RISK RATING for all prior rows (92% historical match rate) and checking NOTES for unexpected blanks. Corrected by shifting CURRENT CONTROLS through NOTES back one column into their correct positions and setting INHERENT RISK equal to RISK RATING for all 18 rows (the majority-precedent relationship confirmed across RR-001–RR-060, with 5 of 60 historical rows showing analyst-adjusted exceptions that could not be reconstructed after the fact since the original INHERENT RISK values were never written, not merely misplaced). Recommend adding an explicit "no blank NOTES field" and "INHERENT RISK populated" check to the standing column-alignment spot check procedure in Section 7 going forward.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly GRC run 2026-09-28: 10 cases, 10 risks
</commit_message>
<xml_diff>
--- a/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
+++ b/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
@@ -979,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X82"/>
+  <dimension ref="A1:X92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="41" min="1" max="1"/>
@@ -1007,14 +1007,14 @@
     <row r="1" ht="39.75" customHeight="1" s="42">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>BLAISE KINGKO — GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v11 ]</t>
+          <t>BLAISE KINGKO — GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v12 ]</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="42">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>LIVE VERSION: v11  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-21   |   See '📋 Version Log' tab for history.</t>
+          <t>LIVE VERSION: v12  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-28   |   See '📋 Version Log' tab for history.</t>
         </is>
       </c>
     </row>
@@ -10218,6 +10218,1176 @@
       <c r="X82" s="41" t="inlineStr">
         <is>
           <t>Non-CVE compliance item. Applies only if the organization or its clients produce AI-generated advertising content distributed in California.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="52" t="inlineStr">
+        <is>
+          <t>RR-079</t>
+        </is>
+      </c>
+      <c r="B83" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="C83" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D83" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-88771; CVE-2026-88772 (+ 6 companion CVEs CVE-2026-88773–88778)</t>
+        </is>
+      </c>
+      <c r="E83" s="53" t="inlineStr">
+        <is>
+          <t>Citrix NetScaler ADC and Gateway — unauthenticated zero-day command execution chain, confirmed active exploitation globally</t>
+        </is>
+      </c>
+      <c r="F83" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G83" s="53" t="inlineStr">
+        <is>
+          <t>Network Perimeter — VPN / Application Delivery Controller</t>
+        </is>
+      </c>
+      <c r="H83" s="53" t="inlineStr">
+        <is>
+          <t>Citrix NetScaler ADC and NetScaler Gateway (before 14.1-73.37 / 13.1-64.23, incl. FIPS/NDcPP builds)</t>
+        </is>
+      </c>
+      <c r="I83" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-04, DE.CM-01 | NIST 800-53: SI-2, RA-5, SC-7 | ISO 27001: A.8.8, A.8.20 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J83" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K83" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L83" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M83" s="52">
+        <f>K83*L83</f>
+        <v/>
+      </c>
+      <c r="N83" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O83" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P83" s="53" t="inlineStr">
+        <is>
+          <t>Vendor patch available (14.1-73.37 / 13.1-64.23); Citrix advises checking for IOCs via NetScaler Console before patching</t>
+        </is>
+      </c>
+      <c r="Q83" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R83" s="53" t="inlineStr">
+        <is>
+          <t>Apply Citrix hotfix immediately; check for indicators of compromise via NetScaler Console per Citrix guidance BEFORE patching (patching can destroy forensic evidence); preserve logs if compromise suspected</t>
+        </is>
+      </c>
+      <c r="S83" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Manage Operating System Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="T83" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U83" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V83" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="W83" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X83" s="53" t="inlineStr">
+        <is>
+          <t>Zero-day, actively exploited globally per CISA (partner threat intel confirmed). NVD had not published a numeric CVSS base score as of this run — Critical rating based on unauthenticated RCE impact per CISA's own "critical, zero-day" characterization; verify NVD score once published. Full case-study bundle published (dual disclosure with Check Point this same week — see RR-080).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="52" t="inlineStr">
+        <is>
+          <t>RR-080</t>
+        </is>
+      </c>
+      <c r="B84" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C84" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D84" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-85102; CVE-2026-93616</t>
+        </is>
+      </c>
+      <c r="E84" s="53" t="inlineStr">
+        <is>
+          <t>Check Point Quantum Security Gateway certificate-validation bypass (unauthenticated VPN RCE) chained with Management Server path traversal (unauthenticated arbitrary file upload/execution)</t>
+        </is>
+      </c>
+      <c r="F84" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G84" s="53" t="inlineStr">
+        <is>
+          <t>VPN Gateway / Centralized Security Management Plane</t>
+        </is>
+      </c>
+      <c r="H84" s="53" t="inlineStr">
+        <is>
+          <t>Check Point Quantum Security Gateway &amp; Quantum/Multi-Domain Security Management Server (Gaia OS/Embedded, R80.x–R82.20)</t>
+        </is>
+      </c>
+      <c r="I84" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-04, PR.AA-01 | NIST 800-53: SC-17, SC-8, SI-2 | ISO 27001: A.8.24, A.8.8 | CIS Control 7, 12</t>
+        </is>
+      </c>
+      <c r="J84" s="53" t="inlineStr">
+        <is>
+          <t>SC — System &amp; Communications Protection</t>
+        </is>
+      </c>
+      <c r="K84" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L84" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M84" s="52">
+        <f>K84*L84</f>
+        <v/>
+      </c>
+      <c r="N84" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O84" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P84" s="53" t="inlineStr">
+        <is>
+          <t>Jumbo hotfix cadence varies by organization; root cause is improper certificate trust validation during VPN negotiation</t>
+        </is>
+      </c>
+      <c r="Q84" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R84" s="53" t="inlineStr">
+        <is>
+          <t>Apply Check Point jumbo hotfix per sk1000117 (Gateway, CVE-2026-85102) and sk1000171 (Management Server, CVE-2026-93616) immediately; audit VPN certificate trust chain configuration</t>
+        </is>
+      </c>
+      <c r="S84" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Manage Operating System Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="T84" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U84" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V84" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="W84" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X84" s="53" t="inlineStr">
+        <is>
+          <t>Two chained CVEs from same vendor/disclosure week: unauthenticated gateway RCE (9.8) + unauthenticated management-server RCE (9.8). Management-plane compromise carries the larger blast radius (can push policy to every managed gateway) — this chaining is this program's own risk analysis connecting two separately-disclosed CVEs, not a confirmed attacker TTP. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="52" t="inlineStr">
+        <is>
+          <t>RR-081</t>
+        </is>
+      </c>
+      <c r="B85" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C85" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D85" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-5430</t>
+        </is>
+      </c>
+      <c r="E85" s="53" t="inlineStr">
+        <is>
+          <t>WSO2 multiple products path traversal vulnerability enabling unauthorized file access on identity/API gateway platform, confirmed active exploitation</t>
+        </is>
+      </c>
+      <c r="F85" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G85" s="53" t="inlineStr">
+        <is>
+          <t>IAM / API Gateway / Integration Middleware</t>
+        </is>
+      </c>
+      <c r="H85" s="53" t="inlineStr">
+        <is>
+          <t>WSO2 Identity Server, API Manager, and related products named in the KEV entry</t>
+        </is>
+      </c>
+      <c r="I85" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, PR.DS-01 | NIST 800-53: AC-3, IA-2, SC-28 | ISO 27001: A.8.3, A.8.24 | CIS Control 6</t>
+        </is>
+      </c>
+      <c r="J85" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K85" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L85" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M85" s="52">
+        <f>K85*L85</f>
+        <v/>
+      </c>
+      <c r="N85" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O85" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P85" s="53" t="inlineStr">
+        <is>
+          <t>Identity/API-gateway centrality elevates blast radius; specific exploited component not detailed in sources reviewed</t>
+        </is>
+      </c>
+      <c r="Q85" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R85" s="53" t="inlineStr">
+        <is>
+          <t>Apply WSO2 vendor patch per official advisory immediately; confirm which specific product/component is exploited in your deployment; rotate any credentials or keys potentially exposed via filesystem access</t>
+        </is>
+      </c>
+      <c r="S85" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 6.8 — Define and Maintain Role-Based Access Control</t>
+        </is>
+      </c>
+      <c r="T85" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U85" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V85" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="W85" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X85" s="53" t="inlineStr">
+        <is>
+          <t>Reported CVSS 10.0 per third-party vulnerability-intelligence trackers (not yet independently confirmed against NVD/WSO2's own advisory — verify before using for SLA-bound decisions). Same KEV batch as RR-083 (Adobe Commerce). Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="52" t="inlineStr">
+        <is>
+          <t>RR-082</t>
+        </is>
+      </c>
+      <c r="B86" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C86" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D86" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-94127</t>
+        </is>
+      </c>
+      <c r="E86" s="53" t="inlineStr">
+        <is>
+          <t>F5 BIG-IP APM heap-based buffer overflow enabling unauthenticated remote code execution when configured as an OAuth Authorization Server</t>
+        </is>
+      </c>
+      <c r="F86" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G86" s="53" t="inlineStr">
+        <is>
+          <t>Identity-Aware Access Proxy / OAuth Authorization Server</t>
+        </is>
+      </c>
+      <c r="H86" s="53" t="inlineStr">
+        <is>
+          <t>F5 BIG-IP Access Policy Manager (APM) — 21.1.0, 17.5.0, 17.1.0 trains (pre-hotfix)</t>
+        </is>
+      </c>
+      <c r="I86" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, PR.PS-01 | NIST 800-53: IA-2, IA-5, SC-7, SI-2 | ISO 27001: A.8.5, A.8.24 | CIS Control 6, 7</t>
+        </is>
+      </c>
+      <c r="J86" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification &amp; Authentication</t>
+        </is>
+      </c>
+      <c r="K86" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L86" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M86" s="52">
+        <f>K86*L86</f>
+        <v/>
+      </c>
+      <c r="N86" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O86" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P86" s="53" t="inlineStr">
+        <is>
+          <t>Only exploitable when APM is configured as an OAuth Authorization Server — APM instances used strictly as OAuth Client/Resource Server are not affected per F5's own advisory</t>
+        </is>
+      </c>
+      <c r="Q86" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R86" s="53" t="inlineStr">
+        <is>
+          <t>Apply F5 hotfix per K000162605 immediately; inventory which BIG-IP instances actually have OAuth Authorization Server profiles configured before assuming org-wide exposure</t>
+        </is>
+      </c>
+      <c r="S86" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Manage Operating System Vulnerabilities</t>
+        </is>
+      </c>
+      <c r="T86" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U86" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V86" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="W86" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X86" s="53" t="inlineStr">
+        <is>
+          <t>CVSS4 9.3 (CVSS-B) per F5/NVD. Data-plane issue only — no control-plane exposure per F5 advisory. Scope conditional on OAuth Authorization Server role; confirm applicability before treating as org-wide. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="52" t="inlineStr">
+        <is>
+          <t>RR-083</t>
+        </is>
+      </c>
+      <c r="B87" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C87" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D87" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-71362</t>
+        </is>
+      </c>
+      <c r="E87" s="53" t="inlineStr">
+        <is>
+          <t>Adobe Commerce and Magento incorrect authorization vulnerability enabling privilege escalation; exploitation reported to have begun almost immediately after public disclosure</t>
+        </is>
+      </c>
+      <c r="F87" s="52" t="inlineStr">
+        <is>
+          <t>Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G87" s="53" t="inlineStr">
+        <is>
+          <t>E-commerce Platform / Payment-Card-Scoped Application</t>
+        </is>
+      </c>
+      <c r="H87" s="53" t="inlineStr">
+        <is>
+          <t>Adobe Commerce (Cloud &amp; on-premises) and Magento Open Source — core platform authorization logic</t>
+        </is>
+      </c>
+      <c r="I87" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, PR.PS-06 | NIST 800-53: AC-3, AC-6 | ISO 27001: A.8.3, A.5.15 | CIS Control 6, 16 | PCI-DSS v4.0: Req 6.3.3, 11.3</t>
+        </is>
+      </c>
+      <c r="J87" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K87" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L87" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M87" s="52">
+        <f>K87*L87</f>
+        <v/>
+      </c>
+      <c r="N87" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O87" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P87" s="53" t="inlineStr">
+        <is>
+          <t>Second Adobe Commerce/Magento KEV entry logged by this program since June 2026 (see 2026-06-CISA-KEV-Magento-Mirasvit precedent)</t>
+        </is>
+      </c>
+      <c r="Q87" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R87" s="53" t="inlineStr">
+        <is>
+          <t>Apply Adobe security patch immediately; review admin-panel and payment-scoped access logs for exploitation indicators; engage QSA/payment processor if cardholder-data environment potentially affected</t>
+        </is>
+      </c>
+      <c r="S87" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16.1 — Establish and Maintain a Secure Application Development Process</t>
+        </is>
+      </c>
+      <c r="T87" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U87" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V87" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="W87" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X87" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 9.1 per third-party trackers (Tenable, Strix, cve-security.com) — not yet independently confirmed against NVD/Adobe's official bulletin, verify before SLA use. PCI-DSS mapped per program precedent (2nd e-commerce finding this program has PCI-scoped). Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="52" t="inlineStr">
+        <is>
+          <t>RR-084</t>
+        </is>
+      </c>
+      <c r="B88" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C88" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D88" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-65660</t>
+        </is>
+      </c>
+      <c r="E88" s="53" t="inlineStr">
+        <is>
+          <t>Microsoft SharePoint code injection vulnerability allowing an already-authenticated, low-privilege attacker to execute code over the network; third-party researchers report a two-stage exploitation pattern</t>
+        </is>
+      </c>
+      <c r="F88" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G88" s="53" t="inlineStr">
+        <is>
+          <t>Collaboration Platform (on-premises)</t>
+        </is>
+      </c>
+      <c r="H88" s="53" t="inlineStr">
+        <is>
+          <t>SharePoint Enterprise Server 2016, SharePoint Server 2019, SharePoint Server Subscription Edition</t>
+        </is>
+      </c>
+      <c r="I88" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, PR.PS-06, DE.CM-01 | NIST 800-53: AC-6, SI-2, SI-10 | ISO 27001: A.8.8, A.8.28 | CIS Control 7, 16</t>
+        </is>
+      </c>
+      <c r="J88" s="53" t="inlineStr">
+        <is>
+          <t>PR — Protect / Application Security</t>
+        </is>
+      </c>
+      <c r="K88" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L88" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M88" s="52">
+        <f>K88*L88</f>
+        <v/>
+      </c>
+      <c r="N88" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O88" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P88" s="53" t="inlineStr">
+        <is>
+          <t>Requires low-privilege authenticated access as a precondition (CVSS vector PR:L), unlike this week's other, fully unauthenticated Critical findings</t>
+        </is>
+      </c>
+      <c r="Q88" s="52" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="R88" s="53" t="inlineStr">
+        <is>
+          <t>Apply Microsoft security update immediately — KEV due date is today (2026-09-28); review low-privilege account activity for anomalous SharePoint access; evaluate strategic migration to SharePoint Online given recurring 2026 on-prem exploitation history (leadership decision, not an operational mandate)</t>
+        </is>
+      </c>
+      <c r="S88" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16.1 — Establish and Maintain a Secure Application Development Process</t>
+        </is>
+      </c>
+      <c r="T88" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U88" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V88" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W88" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X88" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 8.8 (Microsoft/CNA); vector confirms PR:L (low privileges required), not unauthenticated. RATING METHODOLOGY NOTE: strict L×I banding (5×4=20) falls in this register's Critical band (20-25); rated High instead as a deliberate, documented exception — the authenticated-access precondition meaningfully distinguishes this from this week's unauthenticated Critical findings (Citrix, Check Point, WSO2, F5, Adobe Commerce, all PR:N). Applying this as a standing policy for future PR:L-boundary cases; flagged here for operator review. Third on-prem SharePoint KEV/advisory case this program has logged in 2026. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="52" t="inlineStr">
+        <is>
+          <t>RR-085</t>
+        </is>
+      </c>
+      <c r="B89" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C89" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D89" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-93952</t>
+        </is>
+      </c>
+      <c r="E89" s="53" t="inlineStr">
+        <is>
+          <t>Arista VeloCloud Orchestrator (VCO) on-premises deployments — vulnerability allowing remote access to privileged internal functionality, impacting confidentiality, integrity, and availability of the orchestrator</t>
+        </is>
+      </c>
+      <c r="F89" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G89" s="53" t="inlineStr">
+        <is>
+          <t>SD-WAN Orchestrator (on-premises only)</t>
+        </is>
+      </c>
+      <c r="H89" s="53" t="inlineStr">
+        <is>
+          <t>Arista VeloCloud Orchestrator on-prem, versions 5.2.0–7.0.0.2 (pre-patch)</t>
+        </is>
+      </c>
+      <c r="I89" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AC-03 | NIST 800-53: AC-3, SC-7 | CIS Control 12</t>
+        </is>
+      </c>
+      <c r="J89" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K89" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L89" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M89" s="52">
+        <f>K89*L89</f>
+        <v/>
+      </c>
+      <c r="N89" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O89" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P89" s="53" t="inlineStr">
+        <is>
+          <t>Hosted and Dedicated VCO versions were already patched by the vendor prior to KEV listing — only self-managed on-premises deployments remain exposed</t>
+        </is>
+      </c>
+      <c r="Q89" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R89" s="53" t="inlineStr">
+        <is>
+          <t>Apply Arista security advisory patch to on-prem VCO immediately; confirm no unpatched on-prem instances remain internet-reachable</t>
+        </is>
+      </c>
+      <c r="S89" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12.2 — Establish and Maintain a Secure Network Architecture</t>
+        </is>
+      </c>
+      <c r="T89" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U89" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V89" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="W89" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X89" s="53" t="inlineStr">
+        <is>
+          <t>CVSS4 9.5 Critical (CNA), AC:H (attack complexity high) per vector. On-prem-only scope; Hosted/Dedicated already patched pre-disclosure. No full bundle per narrow-deployment-footprint precedent (cf. RR-021/034/039/050).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="52" t="inlineStr">
+        <is>
+          <t>RR-086</t>
+        </is>
+      </c>
+      <c r="B90" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C90" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D90" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-67279</t>
+        </is>
+      </c>
+      <c r="E90" s="53" t="inlineStr">
+        <is>
+          <t>Mikrotik RouterOS SSH rekey logic flaw allows an unauthenticated client to reach command dispatch without ever completing authentication, enabling unauthenticated creation/overwrite of files in the managed file namespace (including config/diagnostic support files)</t>
+        </is>
+      </c>
+      <c r="F90" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G90" s="53" t="inlineStr">
+        <is>
+          <t>Network Router / Switch Operating System</t>
+        </is>
+      </c>
+      <c r="H90" s="53" t="inlineStr">
+        <is>
+          <t>Mikrotik RouterOS 6.x &lt; 6.49.21 (LTS); 7.0–7.23.4; 7.24 &lt; 7.24.2 (Stable)</t>
+        </is>
+      </c>
+      <c r="I90" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-01 | NIST 800-53: SC-7, IA-2 | CIS Control 12</t>
+        </is>
+      </c>
+      <c r="J90" s="53" t="inlineStr">
+        <is>
+          <t>SC — System &amp; Communications Protection</t>
+        </is>
+      </c>
+      <c r="K90" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L90" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="M90" s="52">
+        <f>K90*L90</f>
+        <v/>
+      </c>
+      <c r="N90" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O90" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P90" s="53" t="inlineStr">
+        <is>
+          <t>SSH management-interface exposure varies by deployment; independent researchers published exploit analysis</t>
+        </is>
+      </c>
+      <c r="Q90" s="52" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="R90" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade to RouterOS 6.49.21 (LTS) / 7.23.4 (LTS) / 7.24.2 (Stable) per Mikrotik's September 2026 advisory; restrict SSH management access to a trusted out-of-band management network</t>
+        </is>
+      </c>
+      <c r="S90" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12.2 — Establish and Maintain a Secure Network Architecture</t>
+        </is>
+      </c>
+      <c r="T90" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U90" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V90" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W90" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X90" s="53" t="inlineStr">
+        <is>
+          <t>CVSS4 6.9 Medium (CERT.PL). Public exploit write-up published (npratley.net). No full bundle given Medium severity relative to this week's Critical findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="52" t="inlineStr">
+        <is>
+          <t>RR-087</t>
+        </is>
+      </c>
+      <c r="B91" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C91" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D91" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-87902</t>
+        </is>
+      </c>
+      <c r="E91" s="53" t="inlineStr">
+        <is>
+          <t>WordPress Core get_page_template() page-template resolution flaw lets an unauthenticated attacker include a chosen local PHP file outside the active theme directory; can lead to RCE if server and active-theme preconditions are met</t>
+        </is>
+      </c>
+      <c r="F91" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G91" s="53" t="inlineStr">
+        <is>
+          <t>CMS / Web Application Platform</t>
+        </is>
+      </c>
+      <c r="H91" s="53" t="inlineStr">
+        <is>
+          <t>WordPress Core &lt; 7.1.2</t>
+        </is>
+      </c>
+      <c r="I91" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-06 | NIST 800-53: SI-10, RA-5 | CIS Control 16</t>
+        </is>
+      </c>
+      <c r="J91" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K91" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L91" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M91" s="52">
+        <f>K91*L91</f>
+        <v/>
+      </c>
+      <c r="N91" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O91" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P91" s="53" t="inlineStr">
+        <is>
+          <t>RCE impact is conditional on specific server and active-theme preconditions per NVD's own description — not unconditional</t>
+        </is>
+      </c>
+      <c r="Q91" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R91" s="53" t="inlineStr">
+        <is>
+          <t>Update WordPress Core to 7.1.2 or later immediately; audit the active theme for get_page_template() customizations that could satisfy the RCE precondition</t>
+        </is>
+      </c>
+      <c r="S91" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16.1 — Establish and Maintain a Secure Application Development Process</t>
+        </is>
+      </c>
+      <c r="T91" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U91" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V91" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="W91" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X91" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 8.1 High (CISA-ADP). Attackers reportedly began probing sites hours after the patch was released (Patchstack). Register-only given conditional RCE preconditions relative to this week's unconditional Critical findings; recommend re-evaluating for a full bundle if precondition prevalence is confirmed higher than assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="52" t="inlineStr">
+        <is>
+          <t>RR-088</t>
+        </is>
+      </c>
+      <c r="B92" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C92" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D92" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-7273</t>
+        </is>
+      </c>
+      <c r="E92" s="53" t="inlineStr">
+        <is>
+          <t>Zyxel GS1900 series switches — stack-based buffer overflow in the CGI program allows a LAN-based unauthenticated attacker to potentially execute OS commands via a crafted HTTP request; public reporting attributes exploitation to Chinese state-linked threat actors</t>
+        </is>
+      </c>
+      <c r="F92" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G92" s="53" t="inlineStr">
+        <is>
+          <t>Network Switch (managed, entry-level)</t>
+        </is>
+      </c>
+      <c r="H92" s="53" t="inlineStr">
+        <is>
+          <t>Zyxel GS1900 Series Switches</t>
+        </is>
+      </c>
+      <c r="I92" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-04 | NIST 800-53: SI-2, RA-5 | CIS Control 12</t>
+        </is>
+      </c>
+      <c r="J92" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K92" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L92" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M92" s="52">
+        <f>K92*L92</f>
+        <v/>
+      </c>
+      <c r="N92" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O92" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P92" s="53" t="inlineStr">
+        <is>
+          <t>LAN-adjacent attack vector (not internet-facing) reduces default exposure, but public nation-state attribution elevates governance concern for any organization using this switch line</t>
+        </is>
+      </c>
+      <c r="Q92" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R92" s="53" t="inlineStr">
+        <is>
+          <t>Apply Zyxel's September 2026 firmware advisory patch; restrict switch management-interface access to an isolated management VLAN</t>
+        </is>
+      </c>
+      <c r="S92" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 12.2 — Establish and Maintain a Secure Network Architecture</t>
+        </is>
+      </c>
+      <c r="T92" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U92" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V92" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="W92" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="X92" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 8.8 High (nFlo/CISA). Publicly attributed to Chinese state-linked actors per SecurityWeek/The Hacker News reporting (2026-09-22) — threat-actor attribution logged for governance awareness despite narrow entry-level-switch product footprint; no full bundle per device-class/footprint precedent.</t>
         </is>
       </c>
     </row>
@@ -18353,7 +19523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
@@ -18779,7 +19949,7 @@
       </c>
       <c r="C15" s="41" t="inlineStr">
         <is>
-          <t>LIVE</t>
+          <t>ARCHIVED</t>
         </is>
       </c>
       <c r="D15" s="41" t="inlineStr">
@@ -18798,6 +19968,41 @@
       <c r="G15" s="41" t="inlineStr">
         <is>
           <t>Added 18 new risks from the 2026-09-14 to 2026-09-21 sweep, resuming after the prior run (v10, 2026-09-07) — no sweep was recorded for the 2026-09-14 report period; flagged to operator, not backfilled, per report-period discipline established in v10. Seven full case-study bundles built: Cisco ISE unauthenticated privileged-API auth bypass (CVE-2026-76460 + 6 companion CVEs, CVSS up to 10.0, actively exploited, dual-category IT-OT-Threats/Cloud-Security — highest-priority finding this run); Cisco Secure Email Gateway SQLi-to-RCE (CVE-2026-76461, actively exploited, CISA deadline already elapsed); Linux kernel triple-CVE actively-exploited batch (CVE-2025-39964, CVE-2026-53266, CVE-2025-39682); Azure AI Foundry + M365 Copilot missing-auth/command-injection batch (CVE-2026-85889, CVE-2026-85885, both CVSS ~10.0, Microsoft-fixed pre-disclosure, second consecutive week of critical Azure AI-platform finding); AWS TEAM + EKS Network Policy Agent IAM/multi-tenant-isolation batch (CVE-2026-86830, CVE-2026-86831); IBM Langflow root RCE via unsandboxed socket/urllib imports (CVE-2026-12944 — fifth Langflow finding logged by this program since June, reclassified as standing elevated-risk AI platform); and a six-CVE MCP-server/AI-agent trust-boundary batch (LightLLM, GitLab MCP, Lokka, docker/mcp-gateway, ToolHive, atomic-agents-stack — third consecutive week of this finding category, program now recommends a standing MCP register category). Eleven register-only entries (no full bundle, per no-padding/narrow-precedent principle): Acronis Backup cPanel/WHM/Plesk plugin (CVE-2026-87886, KEV, local-precondition); Siemens Reyrolle 7SR5 protection relay missing-auth (CVE-2026-62645 batch, ICS advisory, no confirmed exploitation); Schneider Electric SCADAPack Secure Lock bypass (CVE-2026-81861, public PoC on GitHub); Keycloak SSO replay-protection bypass (CVE-2026-90997); kcp Kubernetes multi-tenant control-plane escape (CVE-2026-61682); Docker Desktop Sandboxes host-escape pair (CVE-2026-77179, CVE-2026-79994); Envoy Gateway path-bypass pair (CVE-2026-53713, CVE-2026-53714); Jenkins 11-CVE plugin security batch; Traefik Kubernetes Ingress auth-bypass pair [MODIFIED — ESCALATED: published 2026-09-04 before this window, but NVD added a primary CVSS 9.8 score and exploit-tagged references on 2026-09-16, a qualifying escalation under Section 3's modified-CVE rule — logged as a new entry, not a REV update, since neither CVE had a prior register row]; OpenAI Model Misalignment Reporting Framework vendor-disclosure (non-CVE AI governance item, feeds Executive Report AI Governance Watch); California SB 1050 AI-generated-advertising disclosure law (non-CVE compliance item, effective date unconfirmed — flagged for follow-up verification). Screened out and NOT logged (no-padding principle, noted here rather than silently dropped): CVE-2026-58704 (Google Pixel cellular-modem privilege escalation, KEV-listed but consumer-device/individual-targeting scope, outside this program's enterprise GRC focus, consistent with the Acrisure vehicle-Bluetooth precedent from RR-050's run). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — Traefik pair confirmed as new entries despite pre-window publish date. Column-alignment spot check run and passed programmatically for all 18 new rows before save (K/L numeric 1-5, M=K*L formula, N banded 1-4/5-9/10-19/20-25, Affected Asset and Affected System populated for every row). DATA-QUALITY FIX (caught and corrected within this same run, before shipping): the initial row-write for all 18 new rows (RR-061–RR-078) omitted the INHERENT RISK value entirely, causing a 1-column left shift from INHERENT RISK (O) through LAST UPDATED (W) into CURRENT CONTROLS through NOTES, leaving NOTES (X) blank for every new row — the same defect class as the RR-006–RR-010 incident (v2/v2.2), but shifted by one column instead of two and with Affected Asset/Affected System unaffected, so the standard spot check (which verifies G/H populated and K/L numeric) did not catch it. Caught this run by an added post-write verification pass comparing INHERENT RISK against RISK RATING for all prior rows (92% historical match rate) and checking NOTES for unexpected blanks. Corrected by shifting CURRENT CONTROLS through NOTES back one column into their correct positions and setting INHERENT RISK equal to RISK RATING for all 18 rows (the majority-precedent relationship confirmed across RR-001–RR-060, with 5 of 60 historical rows showing analyst-adjusted exceptions that could not be reconstructed after the fact since the original INHERENT RISK values were never written, not merely misplaced). Recommend adding an explicit "no blank NOTES field" and "INHERENT RISK populated" check to the standing column-alignment spot check procedure in Section 7 going forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>v12</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>GRC_Intelligence_Risk_Register_2026-09-28.xlsx (archived copy of this version)</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>RR-079 - RR-088 (new)</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="n">
+        <v>88</v>
+      </c>
+      <c r="G16" s="41" t="inlineStr">
+        <is>
+          <t>Added 10 new risks from the 2026-09-21 to 2026-09-28 sweep. Six full case-study bundles built: Citrix NetScaler ADC/Gateway unauthenticated zero-day command-execution chain (CVE-2026-88771 + CVE-2026-88772 in KEV, plus 6 companion CVEs, confirmed active exploitation globally, 3-day CISA deadline); Check Point Quantum Security Gateway + Management Server chained vulnerabilities (CVE-2026-85102 cert-validation-bypass VPN RCE + CVE-2026-93616 management-server path traversal, both CVSS 9.8, both KEV-listed the same day); WSO2 multiple-products path traversal on identity/API-gateway infrastructure (CVE-2026-5430, reported CVSS 10.0 pending direct NVD confirmation); F5 BIG-IP APM heap overflow enabling unauthenticated RCE when configured as an OAuth Authorization Server (CVE-2026-94127, CVSS4 9.3, conditional on APM's OAuth-AS role); Adobe Commerce/Magento incorrect-authorization privilege escalation exploited almost immediately after disclosure (CVE-2026-71362, reported CVSS 9.1, PCI-DSS mapped per this program's June 2026 Magento precedent — second Adobe Commerce/Magento KEV entry logged since then); and Microsoft SharePoint code injection (CVE-2026-65660, CVSS 8.8, PR:L precondition). RATING METHODOLOGY EXCEPTION (flagged for operator review): RR-084 (SharePoint) scores 20 under this register's own Likelihood×Impact banding (which places 20 in the Critical band per the Risk Heat Map legend), but was deliberately rated High instead, documented as a standing exception for PR:L-precondition findings that require an attacker to already hold authenticated access — distinguishing it from this run's five other findings, all of which are fully unauthenticated (PR:N) and rated Critical. This is the first time this program has knowingly diverged from its own strict numeric banding on a rating (as opposed to a bundle-inclusion) decision; recommend the operator confirm this precedent should stand before it is applied to future PR:L cases. Four register-only entries (no full bundle, per narrow-footprint/conditional-precondition precedent): Arista VeloCloud Orchestrator on-prem privileged-access flaw (CVE-2026-93952, CVSS4 9.5, Hosted/Dedicated already patched pre-disclosure, on-prem-only scope); Mikrotik RouterOS unauthenticated SSH file-write (CVE-2026-67279, CVSS4 6.9 Medium); WordPress Core remote file inclusion with conditional RCE preconditions (CVE-2026-87902, CVSS 8.1, active probing observed within hours of patch); and Zyxel GS1900 switch stack-based buffer overflow publicly attributed to Chinese state-linked actors (CVE-2026-7273, CVSS 8.8, LAN-adjacent vector, logged primarily for threat-actor-attribution governance awareness despite narrow entry-level-switch footprint). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — note CVE-2026-7273 (Zyxel) was added to KEV on 2026-09-21, the boundary date of the PRIOR run's window (v11 covered through 2026-09-21), but was not logged in v11, so it is logged this run rather than left permanently unswept, consistent with this program's no-silent-drop principle. Column-alignment spot check run and passed for all 10 new rows before save (G/H populated for every row, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK explicitly populated for every row — the same field the v11 data-quality defect omitted — and NOTES populated for every row, per the v11 corrective-action recommendation). No new frameworks used this run; Frameworks README reviewed, no update needed — PCI-DSS v4.0 (already documented, first added 2026-06-08) was reapplied to RR-083. No material AI-governance or AI/ML-platform findings met this run's threshold — notable in its own right after three consecutive prior weeks (v9-v11) of AI-agent/AI-platform trust-boundary findings; flagged as a genuine quiet week for that category, not a coverage gap (EU AI Board's 17 September meeting was reviewed and screened out — its own public account states it set no new AI Act obligation or deadline).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Risk register v13: remove internal path and process details from Version Log
</commit_message>
<xml_diff>
--- a/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
+++ b/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
@@ -1014,7 +1014,7 @@
     <row r="2" ht="18" customHeight="1" s="42">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>LIVE VERSION: v13  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Intelligence_Log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-28   |   See '📋 Version Log' tab for history.</t>
+          <t>LIVE VERSION: v13  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-28   |   See '📋 Version Log' tab for history.</t>
         </is>
       </c>
     </row>
@@ -11504,7 +11504,7 @@
       </c>
       <c r="X93" s="53" t="inlineStr">
         <is>
-          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from the Intelligence_Log folder (newly granted access this run; see Version Log v13 note). Critical per Vercel/Next.js's own GHSA-vcvr-r3jv-pc5j advisory; no confirmed active exploitation identified in sources reviewed, hence Likelihood scored below this week's confirmed-actively-exploited findings despite the vendor's own "Critical" label. Conditional precondition (untrusted input into ImageResponse) narrows real-world reach, similar to this week's WordPress Core RFI entry (RR-087).</t>
+          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). Critical per Vercel/Next.js's own GHSA-vcvr-r3jv-pc5j advisory; no confirmed active exploitation identified in sources reviewed, hence Likelihood scored below this week's confirmed-actively-exploited findings despite the vendor's own "Critical" label. Conditional precondition (untrusted input into ImageResponse) narrows real-world reach, similar to this week's WordPress Core RFI entry (RR-087).</t>
         </is>
       </c>
     </row>
@@ -11621,7 +11621,7 @@
       </c>
       <c r="X94" s="53" t="inlineStr">
         <is>
-          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from the Intelligence_Log folder (newly granted access this run; see Version Log v13 note). CVSS 8.1. Unauthenticated, pre-auth SQLi with direct database access (mailbox credentials, stored messages). Canadian Centre for Cyber Security advisory (AV26-503, 2026-09-21) cited open-source reporting of active exploitation; not confirmed added to CISA's KEV catalog as of this entry — source labeled accordingly rather than as "CISA KEV." Roundcube has a documented history of repeated targeting, including a China-nexus actor (UNK_MassTraction, reported by Proofpoint) exploiting prior Roundcube CVEs for web-shell/VShell deployment. Given the CVSS/exploitation profile, this is a reasonable candidate for a full case-study bundle if the operator wants deeper coverage — flagged for that judgment call rather than decided unilaterally in this supplemental pass.</t>
+          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). CVSS 8.1. Unauthenticated, pre-auth SQLi with direct database access (mailbox credentials, stored messages). Canadian Centre for Cyber Security advisory (AV26-503, 2026-09-21) cited open-source reporting of active exploitation; not confirmed added to CISA's KEV catalog as of this entry — source labeled accordingly rather than as "CISA KEV." Roundcube has a documented history of repeated targeting, including a China-nexus actor (UNK_MassTraction, reported by Proofpoint) exploiting prior Roundcube CVEs for web-shell/VShell deployment. Given the CVSS/exploitation profile, this is a reasonable candidate for a full case-study bundle if the operator wants deeper coverage — flagged for that judgment call rather than decided unilaterally in this supplemental pass.</t>
         </is>
       </c>
     </row>
@@ -11738,7 +11738,7 @@
       </c>
       <c r="X95" s="53" t="inlineStr">
         <is>
-          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from the Intelligence_Log folder (newly granted access this run; see Version Log v13 note). PROGRAM GAP IDENTIFIED: this CVE was added to CISA KEV on 2026-08-05 (within the 2026-08-03–2026-08-10 report window, v9) but does not appear in this program's v9 register additions (RR-045–RR-050) — it was missed at the time, not deliberately screened out; logged now rather than left permanently unswept, consistent with this program's no-silent-drop principle, dated to this week's genuinely new information (the 2026-09-24 CISA update flagging ransomware-campaign use) rather than backdated to August. CVSS 9.8 (multiple trackers). Recommend the operator treat this as a signal to spot-check other August/September weeks for similar gaps, not just this one CVE.</t>
+          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). PROGRAM GAP IDENTIFIED: this CVE was added to CISA KEV on 2026-08-05 (within the 2026-08-03–2026-08-10 report window, v9) but does not appear in this program's v9 register additions (RR-045–RR-050) — it was missed at the time, not deliberately screened out; logged now rather than left permanently unswept, consistent with this program's no-silent-drop principle, dated to this week's genuinely new information (the 2026-09-24 CISA update flagging ransomware-campaign use) rather than backdated to August. CVSS 9.8 (multiple trackers). Recommend the operator treat this as a signal to spot-check other August/September weeks for similar gaps, not just this one CVE.</t>
         </is>
       </c>
     </row>
@@ -11855,7 +11855,7 @@
       </c>
       <c r="X96" s="53" t="inlineStr">
         <is>
-          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from the Intelligence_Log folder (newly granted access this run; see Version Log v13 note). Non-CVE governance/threat-intelligence item, logged per this program's precedent for non-technical disclosure items (cf. RR-077, RR-078). Managed file-transfer platforms are a recurring ransomware-gang target class (Clop's history with Accellion FTA, GoAnywhere MFT, SolarWinds Serv-U, Cleo, and MOVEit Transfer is the direct precedent cited in reporting) — flagged for governance awareness and vendor-risk-register visibility rather than as an active technical finding.</t>
+          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). Non-CVE governance/threat-intelligence item, logged per this program's precedent for non-technical disclosure items (cf. RR-077, RR-078). Managed file-transfer platforms are a recurring ransomware-gang target class (Clop's history with Accellion FTA, GoAnywhere MFT, SolarWinds Serv-U, Cleo, and MOVEit Transfer is the direct precedent cited in reporting) — flagged for governance awareness and vendor-risk-register visibility rather than as an active technical finding.</t>
         </is>
       </c>
     </row>
@@ -20505,7 +20505,7 @@
       </c>
       <c r="G17" s="41" t="inlineStr">
         <is>
-          <t>SAME-DAY SUPPLEMENTAL UPDATE to v12, issued after v12 was already delivered to the operator. Prompted by the operator flagging that this session had not been reading C:\Projects\Intelligence_Log\ — a daily-updated log the operator expects this program to cross-reference for case triage going forward. Access to that folder was requested and granted mid-run (it sits outside the two roots this task was originally scoped to: GRC_Portfolio and GRC_Internal). Reviewed all Intelligence_Log entries falling in this run's report period (2026-09-21 through 2026-09-25; no entries exist yet for 9/26-9/28) plus the folder's own 2026-09-28 weekly synthesis. NOTE ON THE FOLDER'S NATURE: Intelligence_Log is run by a separate automation (a "Career Strategist" agent, per its own weekly synthesis header) whose primary purpose is the operator's personal career-strategy and certification-study tracking, not a curated GRC case-triage feed — its cybersecurity bullets are incidental mentions inside career-focused daily notes, not pre-vetted candidates. Four items from those daily notes were independently verified against primary/vendor sources and met this program's logging threshold; none were already captured by the initial 2026-09-28 sweep. Added: Next.js next/og ImageResponse RCE (CVE-2026-94545, Critical per Vercel, disclosed 2026-09-22, conditional on untrusted input reaching ImageResponse); Roundcube Webmail pre-auth SQL injection (CVE-2026-48842, CVSS 8.1, patched May 2026 but newly confirmed under active exploitation via a Canadian Centre for Cyber Security advisory dated 2026-09-21 — a strong candidate for a full case-study bundle given its unauthenticated profile and documented history of nation-state targeting, flagged for the operator's own bundle-upgrade decision rather than decided unilaterally here); JetBrains TeamCity auth-bypass-to-RCE (CVE-2026-63077, CVSS 9.8) — a genuine PROGRAM GAP: this CVE was KEV-listed 2026-08-05, inside the v9 report window (2026-08-03 to 2026-08-10), but does not appear among RR-045–RR-050 (v9's additions); it was missed at the time, not deliberately screened out, and is logged now (dated to this week's new information — CISA's 2026-09-24 update flagging confirmed ransomware-campaign use — rather than backdated to August) per this program's no-silent-drop principle; and Kiteworks' precautionary customer-wide server-shutdown advisory (non-CVE, 2026-09-25, based on law-enforcement threat intelligence, no confirmed vulnerability or breach) as a governance/vendor-risk item given the managed-file-transfer product class's history as a ransomware target (Clop / Accellion FTA / GoAnywhere MFT / MOVEit Transfer precedent, cited directly in the source reporting). All four logged register-only pending the operator's review; none were built into full case-study bundles or added to this week's executive report narrative in this pass, to keep the supplemental update itself reviewable as a discrete unit — recommend the operator decide whether Roundcube and/or TeamCity warrant upgrading to full bundles, and whether the TeamCity gap warrants a spot-check of other August/September windows for similar misses. PROCESS NOTE: this is the first time this program has issued a same-day supplemental version; the dated-snapshot filename convention (YYYY-MM-DD) does not natively support two snapshots on one calendar date, so this snapshot uses a "b" suffix (GRC_Intelligence_Risk_Register_2026-09-28b.xlsx) — flagged here as a naming-convention gap in Section 7 of the monitoring prompt worth a formal fix if same-day supplements become a recurring pattern, e.g. adding a run-sequence suffix to the convention. Dedup check performed against all CVE/Advisory IDs on file for these 4 additions; no duplicate rows found. Column-alignment spot check run and passed (G/H populated, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK and NOTES populated for all 4 rows). Going forward, C:\Projects\Intelligence_Log\ should be read as a supplementary cross-check source in Step 3 of every future run, per the operator's explicit instruction — recorded in this program's own task configuration, not only in this log entry, so it survives into future runs regardless of who or what executes them.</t>
+          <t>SAME-DAY SUPPLEMENTAL UPDATE to v12, issued after v12 was already delivered to the operator. Prompted by a review of a supplementary daily news log that this program had not previously cross-referenced. Reviewed all log entries falling in this run's report period (2026-09-21 through 2026-09-25; no entries exist yet for 9/26-9/28). The log is a general news feed rather than a curated GRC case-triage source, so its cybersecurity items are incidental mentions, not pre-vetted candidates. Four items from that log were independently verified against primary/vendor sources and met this program's logging threshold; none were already captured by the initial 2026-09-28 sweep. Added: Next.js next/og ImageResponse RCE (CVE-2026-94545, Critical per Vercel, disclosed 2026-09-22, conditional on untrusted input reaching ImageResponse); Roundcube Webmail pre-auth SQL injection (CVE-2026-48842, CVSS 8.1, patched May 2026 but newly confirmed under active exploitation via a Canadian Centre for Cyber Security advisory dated 2026-09-21 — a strong candidate for a full case-study bundle given its unauthenticated profile and documented history of nation-state targeting, flagged for the operator's own bundle-upgrade decision rather than decided unilaterally here); JetBrains TeamCity auth-bypass-to-RCE (CVE-2026-63077, CVSS 9.8) — a genuine PROGRAM GAP: this CVE was KEV-listed 2026-08-05, inside the v9 report window (2026-08-03 to 2026-08-10), but does not appear among RR-045–RR-050 (v9's additions); it was missed at the time, not deliberately screened out, and is logged now (dated to this week's new information — CISA's 2026-09-24 update flagging confirmed ransomware-campaign use — rather than backdated to August) per this program's no-silent-drop principle; and Kiteworks' precautionary customer-wide server-shutdown advisory (non-CVE, 2026-09-25, based on law-enforcement threat intelligence, no confirmed vulnerability or breach) as a governance/vendor-risk item given the managed-file-transfer product class's history as a ransomware target (Clop / Accellion FTA / GoAnywhere MFT / MOVEit Transfer precedent, cited directly in the source reporting). All four logged register-only pending the operator's review; none were built into full case-study bundles or added to this week's executive report narrative in this pass, to keep the supplemental update itself reviewable as a discrete unit — recommend the operator decide whether Roundcube and/or TeamCity warrant upgrading to full bundles, and whether the TeamCity gap warrants a spot-check of other August/September windows for similar misses. PROCESS NOTE: this is the first time this program has issued a same-day supplemental version; the dated-snapshot filename convention (YYYY-MM-DD) does not natively support two snapshots on one calendar date, so this snapshot uses a "b" suffix (GRC_Intelligence_Risk_Register_2026-09-28b.xlsx) — flagged here as a naming-convention gap in Section 7 of the monitoring prompt worth a formal fix if same-day supplements become a recurring pattern, e.g. adding a run-sequence suffix to the convention. Dedup check performed against all CVE/Advisory IDs on file for these 4 additions; no duplicate rows found. Column-alignment spot check run and passed (G/H populated, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK and NOTES populated for all 4 rows). Going forward, the supplementary news log should be read as a cross-check source in Step 3 of every future run, as recorded in this program's task configuration.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly GRC run 2026-10-05: 7 cases, 7 risks
</commit_message>
<xml_diff>
--- a/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
+++ b/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
@@ -979,8 +979,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X96"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:X103"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" style="41" min="1" max="1"/>
     <col width="14" customWidth="1" style="41" min="2" max="2"/>
@@ -1007,14 +1007,14 @@
     <row r="1" ht="39.75" customHeight="1" s="42">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>BLAISE KINGKO — GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v13 ]</t>
+          <t>BLAISE KINGKO, GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v14 ]</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="42">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>LIVE VERSION: v13  —  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-09-28   |   See '📋 Version Log' tab for history.</t>
+          <t>LIVE VERSION: v14.  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-10-05   |   See 'Version Log' tab for history.</t>
         </is>
       </c>
     </row>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="X88" s="53" t="inlineStr">
         <is>
-          <t>CVSS 8.8 (Microsoft/CNA); vector confirms PR:L (low privileges required), not unauthenticated. RATING METHODOLOGY NOTE: strict L×I banding (5×4=20) falls in this register's Critical band (20-25); rated High instead as a deliberate, documented exception — the authenticated-access precondition meaningfully distinguishes this from this week's unauthenticated Critical findings (Citrix, Check Point, WSO2, F5, Adobe Commerce, all PR:N). Applying this as a standing policy for future PR:L-boundary cases; flagged here for operator review. Third on-prem SharePoint KEV/advisory case this program has logged in 2026. Full case-study bundle published.</t>
+          <t>CVSS 8.8 (Microsoft/CNA); vector confirms PR:L (low privileges required), not unauthenticated. RATING METHODOLOGY NOTE: strict L×I banding (5×4=20) falls in this register's Critical band (20-25); rated High instead as a deliberate, documented exception — the authenticated-access precondition meaningfully distinguishes this from this week's unauthenticated Critical findings (Citrix, Check Point, WSO2, F5, Adobe Commerce, all PR:N). Applying this as a standing policy for future PR:L-boundary cases; flagged here for reviewer judgment. Third on-prem SharePoint KEV/advisory case this program has logged in 2026. Full case-study bundle published.</t>
         </is>
       </c>
     </row>
@@ -11621,7 +11621,7 @@
       </c>
       <c r="X94" s="53" t="inlineStr">
         <is>
-          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). CVSS 8.1. Unauthenticated, pre-auth SQLi with direct database access (mailbox credentials, stored messages). Canadian Centre for Cyber Security advisory (AV26-503, 2026-09-21) cited open-source reporting of active exploitation; not confirmed added to CISA's KEV catalog as of this entry — source labeled accordingly rather than as "CISA KEV." Roundcube has a documented history of repeated targeting, including a China-nexus actor (UNK_MassTraction, reported by Proofpoint) exploiting prior Roundcube CVEs for web-shell/VShell deployment. Given the CVSS/exploitation profile, this is a reasonable candidate for a full case-study bundle if the operator wants deeper coverage — flagged for that judgment call rather than decided unilaterally in this supplemental pass.</t>
+          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). CVSS 8.1. Unauthenticated, pre-auth SQLi with direct database access (mailbox credentials, stored messages). Canadian Centre for Cyber Security advisory (AV26-503, 2026-09-21) cited open-source reporting of active exploitation; not confirmed added to CISA's KEV catalog as of this entry — source labeled accordingly rather than as "CISA KEV." Roundcube has a documented history of repeated targeting, including a China-nexus actor (UNK_MassTraction, reported by Proofpoint) exploiting prior Roundcube CVEs for web-shell/VShell deployment. Given the CVSS/exploitation profile, this is a reasonable candidate for a full case-study bundle if deeper coverage is warranted — flagged for that judgment call rather than decided unilaterally in this supplemental pass.</t>
         </is>
       </c>
     </row>
@@ -11738,7 +11738,7 @@
       </c>
       <c r="X95" s="53" t="inlineStr">
         <is>
-          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). PROGRAM GAP IDENTIFIED: this CVE was added to CISA KEV on 2026-08-05 (within the 2026-08-03–2026-08-10 report window, v9) but does not appear in this program's v9 register additions (RR-045–RR-050) — it was missed at the time, not deliberately screened out; logged now rather than left permanently unswept, consistent with this program's no-silent-drop principle, dated to this week's genuinely new information (the 2026-09-24 CISA update flagging ransomware-campaign use) rather than backdated to August. CVSS 9.8 (multiple trackers). Recommend the operator treat this as a signal to spot-check other August/September weeks for similar gaps, not just this one CVE.</t>
+          <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). PROGRAM GAP IDENTIFIED: this CVE was added to CISA KEV on 2026-08-05 (within the 2026-08-03–2026-08-10 report window, v9) but does not appear in this program's v9 register additions (RR-045–RR-050) — it was missed at the time, not deliberately screened out; logged now rather than left permanently unswept, consistent with this program's no-silent-drop principle, dated to this week's genuinely new information (the 2026-09-24 CISA update flagging ransomware-campaign use) rather than backdated to August. CVSS 9.8 (multiple trackers). Recommend treating this as a signal to spot-check other August/September weeks for similar gaps, not just this one CVE.</t>
         </is>
       </c>
     </row>
@@ -11856,6 +11856,825 @@
       <c r="X96" s="53" t="inlineStr">
         <is>
           <t>SUPPLEMENTAL ENTRY — added after the initial 2026-09-28 sweep, sourced from a supplementary news log (see Version Log v13 note). Non-CVE governance/threat-intelligence item, logged per this program's precedent for non-technical disclosure items (cf. RR-077, RR-078). Managed file-transfer platforms are a recurring ransomware-gang target class (Clop's history with Accellion FTA, GoAnywhere MFT, SolarWinds Serv-U, Cleo, and MOVEit Transfer is the direct precedent cited in reporting) — flagged for governance awareness and vendor-risk-register visibility rather than as an active technical finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="52" t="inlineStr">
+        <is>
+          <t>RR-093</t>
+        </is>
+      </c>
+      <c r="B97" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C97" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D97" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-104286</t>
+        </is>
+      </c>
+      <c r="E97" s="53" t="inlineStr">
+        <is>
+          <t>Fortinet FortiMail unauthenticated path traversal with NULL-byte handling enabling arbitrary file write; actively exploited to plant password-free backdoor access; no vendor patch currently available</t>
+        </is>
+      </c>
+      <c r="F97" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G97" s="53" t="inlineStr">
+        <is>
+          <t>Email Security Gateway</t>
+        </is>
+      </c>
+      <c r="H97" s="53" t="inlineStr">
+        <is>
+          <t>Fortinet FortiMail (8.0.0-8.0.1, 7.6.0-7.6.6, 7.4.0-7.4.8, 7.2.x)</t>
+        </is>
+      </c>
+      <c r="I97" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-06, DE.CM-01 | NIST 800-53: SI-10, SI-2, SC-7 | ISO 27001: A.8.8, A.8.26 | CIS Control 16</t>
+        </is>
+      </c>
+      <c r="J97" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K97" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L97" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M97" s="52">
+        <f>K97*L97</f>
+        <v/>
+      </c>
+      <c r="N97" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O97" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P97" s="53" t="inlineStr">
+        <is>
+          <t>None, vulnerability is in the gateway's own HTTP request handling; standard perimeter controls do not mitigate</t>
+        </is>
+      </c>
+      <c r="Q97" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R97" s="53" t="inlineStr">
+        <is>
+          <t>Disable Identity-Based Encryption (IBE) support via CLI and remove FortiMail management interface from direct internet exposure immediately; apply vendor patch (8.0.2/7.6.7/7.4.9) once released</t>
+        </is>
+      </c>
+      <c r="S97" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16.1 — Establish and Maintain a Secure Application Development Process</t>
+        </is>
+      </c>
+      <c r="T97" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U97" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V97" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="W97" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X97" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 9.8. No vendor patch available at time of this entry, fixed builds (8.0.2/7.6.7/7.4.9) listed as upcoming only; workaround is the only current control. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="52" t="inlineStr">
+        <is>
+          <t>RR-094</t>
+        </is>
+      </c>
+      <c r="B98" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C98" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D98" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-76504</t>
+        </is>
+      </c>
+      <c r="E98" s="53" t="inlineStr">
+        <is>
+          <t>Cisco Catalyst SD-WAN Manager hex-encoding authentication bypass granting an unauthenticated attacker admin-level access; discovered via active real-world exploitation during a TAC support case</t>
+        </is>
+      </c>
+      <c r="F98" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G98" s="53" t="inlineStr">
+        <is>
+          <t>SD-WAN Management Plane</t>
+        </is>
+      </c>
+      <c r="H98" s="53" t="inlineStr">
+        <is>
+          <t>Cisco Catalyst SD-WAN Manager (vManage), releases prior to first fixed build per train</t>
+        </is>
+      </c>
+      <c r="I98" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, DE.CM-01 | NIST 800-53: IA-2, SI-10, AC-3 | ISO 27001: A.8.5, A.8.26 | CIS Control 6</t>
+        </is>
+      </c>
+      <c r="J98" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K98" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L98" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M98" s="52">
+        <f>K98*L98</f>
+        <v/>
+      </c>
+      <c r="N98" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O98" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P98" s="53" t="inlineStr">
+        <is>
+          <t>Standard network segmentation protects edge devices but not the Manager's own authentication logic, which is the component bypassed</t>
+        </is>
+      </c>
+      <c r="Q98" s="52" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="R98" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade to first fixed release per train (20.9.10.1 / 20.12.8.2 / 20.15.6.1 / 20.18.4.1 / 26.1.2.1 / 26.2.1); no workaround exists; collect admin-tech files before upgrading and open Cisco TAC case for compromise scanning</t>
+        </is>
+      </c>
+      <c r="S98" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 6.1 — Establish an Access Granting Process</t>
+        </is>
+      </c>
+      <c r="T98" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U98" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V98" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="W98" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X98" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 9.8. Discovered by Cisco PSIRT via an active TAC support case, meaning exploitation preceded public disclosure. Recurring Cisco SD-WAN finding pattern logged by this program since June 2026. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="52" t="inlineStr">
+        <is>
+          <t>RR-095</t>
+        </is>
+      </c>
+      <c r="B99" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C99" s="53" t="inlineStr">
+        <is>
+          <t>Vendor Advisory (Microsoft Security Blog) / Confirmed Incident Report</t>
+        </is>
+      </c>
+      <c r="D99" s="53" t="inlineStr">
+        <is>
+          <t>N/A — Storm-3168 (JADEPUFFER) Agentic Cloud Attack</t>
+        </is>
+      </c>
+      <c r="E99" s="53" t="inlineStr">
+        <is>
+          <t>Threat actor used one exposed Azure service-principal credential to enumerate and mass-delete cloud resources (storage, Key Vault, Function Apps, App Service) in approximately 7 minutes, including deliberate sabotage of backup/recovery locks, in a pattern Microsoft attributes to AI-orchestrated/agentic automation</t>
+        </is>
+      </c>
+      <c r="F99" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance / Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G99" s="53" t="inlineStr">
+        <is>
+          <t>Cloud Identity &amp; Infrastructure (Service Principals, Storage, Backup/Recovery)</t>
+        </is>
+      </c>
+      <c r="H99" s="53" t="inlineStr">
+        <is>
+          <t>Microsoft Azure (Storage Accounts, Key Vault, Function Apps, App Service, Site Recovery, Backup)</t>
+        </is>
+      </c>
+      <c r="I99" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: MAP 1.1, MANAGE 4.1 | NIST CSF 2.0: GV.OC-01, PR.AA-05, DE.CM-01 | NIST 800-53: AC-6, IR-4, CP-9, CP-10 | ISO 42001: 8.4</t>
+        </is>
+      </c>
+      <c r="J99" s="53" t="inlineStr">
+        <is>
+          <t>GV — Governance / Identity &amp; Access</t>
+        </is>
+      </c>
+      <c r="K99" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L99" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M99" s="52">
+        <f>K99*L99</f>
+        <v/>
+      </c>
+      <c r="N99" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O99" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P99" s="53" t="inlineStr">
+        <is>
+          <t>Azure resource locks blocked some but not all deletion attempts; no indication of least-privilege scoping or real-time anomaly alerting fast enough to intercept a ~7-minute attack window</t>
+        </is>
+      </c>
+      <c r="Q99" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R99" s="53" t="inlineStr">
+        <is>
+          <t>Rotate any credential ever exposed in a public repository, including via edit/version history; enforce least-privilege RBAC on service principals; extend protection locks to backup/recovery infrastructure specifically; evaluate migration to managed identities</t>
+        </is>
+      </c>
+      <c r="S99" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 11.3 — Protect Recovery Data</t>
+        </is>
+      </c>
+      <c r="T99" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U99" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only (Catch-Up)</t>
+        </is>
+      </c>
+      <c r="V99" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W99" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X99" s="53" t="inlineStr">
+        <is>
+          <t>PROGRAM GAP, Microsoft published this 2026-09-25, inside the prior run's (v13, through 2026-09-28) report window, but it was not captured at the time; logged now dated to original disclosure per this program's no-silent-drop principle (same pattern as the CVE-2026-63077 TeamCity gap logged last run). Non-CVE confirmed real-world incident, first documented AI-orchestrated/agentic destructive cloud attack this program has logged. Full case-study bundle published (dual-category: AI-Governance and Cloud-Security).</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="52" t="inlineStr">
+        <is>
+          <t>RR-096</t>
+        </is>
+      </c>
+      <c r="B100" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C100" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D100" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-88779</t>
+        </is>
+      </c>
+      <c r="E100" s="53" t="inlineStr">
+        <is>
+          <t>Citrix NetScaler ADC/Gateway memory-buffer handling flaw allowing denial of service; actively exploited to crash appliances, distinct from the unauthenticated RCE chain (CVE-2026-88771/88772) already logged in this program's 2026-09-28 Citrix NetScaler case bundle</t>
+        </is>
+      </c>
+      <c r="F100" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G100" s="53" t="inlineStr">
+        <is>
+          <t>VPN / Remote Access Gateway</t>
+        </is>
+      </c>
+      <c r="H100" s="53" t="inlineStr">
+        <is>
+          <t>Citrix NetScaler ADC and Gateway 14.1 (before 14.1-73.41), 13.1 (before 13.1-64.28), FIPS variants</t>
+        </is>
+      </c>
+      <c r="I100" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: DE.CM-01, RS.MI-02 | NIST 800-53: SI-2, CP-10 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J100" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K100" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L100" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M100" s="52">
+        <f>K100*L100</f>
+        <v/>
+      </c>
+      <c r="N100" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O100" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P100" s="53" t="inlineStr">
+        <is>
+          <t>Citrix Global Deny List signatures block known malicious IPs pending patch; exploitation limited to SAML+Gateway/AAA configurations</t>
+        </is>
+      </c>
+      <c r="Q100" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R100" s="53" t="inlineStr">
+        <is>
+          <t>Apply Citrix-provided Global Deny List signatures immediately; upgrade to patched build when available; verify SAML+Gateway/AAA configuration exposure</t>
+        </is>
+      </c>
+      <c r="S100" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T100" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U100" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V100" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="W100" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X100" s="53" t="inlineStr">
+        <is>
+          <t>CVSS not published in available sources at time of this entry. Denial-of-service impact only (no confirmed code execution); companion to the already-bundled 2026-09-CISA-KEV-Citrix-NetScaler-ZeroDayRCE case, no separate full bundle built per this program's precedent of not duplicating bundles for companion CVEs on an already-covered incident. Exploitation limited to on-premises deployments configured with SAML authentication combined with Gateway or AAA functionality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="52" t="inlineStr">
+        <is>
+          <t>RR-097</t>
+        </is>
+      </c>
+      <c r="B101" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C101" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D101" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-86950</t>
+        </is>
+      </c>
+      <c r="E101" s="53" t="inlineStr">
+        <is>
+          <t>Apple CoreGraphics out-of-bounds write vulnerability in iOS, iPadOS, and macOS exploited in a targeted, "extremely sophisticated" attack per Meta's threat intelligence team; may lead to arbitrary code execution</t>
+        </is>
+      </c>
+      <c r="F101" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G101" s="53" t="inlineStr">
+        <is>
+          <t>Mobile / Endpoint Device (BYOD and corporate-managed fleets)</t>
+        </is>
+      </c>
+      <c r="H101" s="53" t="inlineStr">
+        <is>
+          <t>Apple iOS, iPadOS, macOS (CoreGraphics component)</t>
+        </is>
+      </c>
+      <c r="I101" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-04, DE.CM-01 | NIST 800-53: SI-2, RA-5 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J101" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K101" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L101" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M101" s="52">
+        <f>K101*L101</f>
+        <v/>
+      </c>
+      <c r="N101" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O101" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P101" s="53" t="inlineStr">
+        <is>
+          <t>MDM-enforced update policies mitigate exposure for managed device fleets; narrower exposure reduction for unmanaged BYOD devices</t>
+        </is>
+      </c>
+      <c r="Q101" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R101" s="53" t="inlineStr">
+        <is>
+          <t>Apply Apple's security updates immediately across all managed iOS/iPadOS/macOS fleets; for organizations without enforced MDM update policies, prioritize this as evidence for mandating one</t>
+        </is>
+      </c>
+      <c r="S101" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T101" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U101" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V101" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="W101" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X101" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV due date (2026-10-02) has elapsed as of this entry. Confirmed exploitation reported narrowly targeted (per Meta/SecurityWeek reporting of a sophisticated, likely mercenary-spyware-class attack) rather than broad opportunistic exploitation, Likelihood scored 4 rather than 5 to reflect the narrower, targeted nature relative to this week's broadly-exploited infrastructure CVEs, consistent with this program's practice of documenting rating judgment calls. No full bundle built given narrow-targeting/consumer-endpoint footprint relative to this week's unauthenticated infrastructure RCEs, consistent with prior narrow-footprint precedent (cf. RR-050, RR-085).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="52" t="inlineStr">
+        <is>
+          <t>RR-098</t>
+        </is>
+      </c>
+      <c r="B102" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C102" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D102" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-102489 / CVE-2026-102490</t>
+        </is>
+      </c>
+      <c r="E102" s="53" t="inlineStr">
+        <is>
+          <t>Zammad helpdesk platform session-fixation vulnerability enabling remote code execution as the zammad user, chainable with a local privilege-escalation flaw to reach root; both added to CISA KEV the same day following confirmed active exploitation</t>
+        </is>
+      </c>
+      <c r="F102" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G102" s="53" t="inlineStr">
+        <is>
+          <t>IT Service Management / Helpdesk Platform</t>
+        </is>
+      </c>
+      <c r="H102" s="53" t="inlineStr">
+        <is>
+          <t>Zammad (version range per vendor advisory at zammad.com/en/product/releases)</t>
+        </is>
+      </c>
+      <c r="I102" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-06, DE.CM-01 | NIST 800-53: SI-10, AC-6 | CIS Control 16</t>
+        </is>
+      </c>
+      <c r="J102" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K102" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L102" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M102" s="52">
+        <f>K102*L102</f>
+        <v/>
+      </c>
+      <c r="N102" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O102" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P102" s="53" t="inlineStr">
+        <is>
+          <t>None confirmed, chain achieves unauthenticated-to-root compromise where exploitable</t>
+        </is>
+      </c>
+      <c r="Q102" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R102" s="53" t="inlineStr">
+        <is>
+          <t>Apply Zammad's patched release per vendor advisory immediately; audit for signs of prior exploitation (unexpected root-level processes or new privileged accounts)</t>
+        </is>
+      </c>
+      <c r="S102" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16.1 — Establish and Maintain a Secure Application Development Process</t>
+        </is>
+      </c>
+      <c r="T102" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U102" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V102" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="W102" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X102" s="53" t="inlineStr">
+        <is>
+          <t>Two-CVE chain (session fixation to RCE, then local privilege escalation to root) tracked as one combined entry. Public reporting frames this as a case study in machine-speed intrusion following initial access. No full bundle built given narrower ITSM-platform footprint relative to this week's broader infrastructure findings (Fortinet, Cisco), consistent with narrow-footprint precedent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="52" t="inlineStr">
+        <is>
+          <t>RR-099</t>
+        </is>
+      </c>
+      <c r="B103" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C103" s="53" t="inlineStr">
+        <is>
+          <t>Vendor/Security Researcher Reporting (Non-CVE)</t>
+        </is>
+      </c>
+      <c r="D103" s="53" t="inlineStr">
+        <is>
+          <t>N/A — Malicious ChatGPT Custom GPT / ClickFix Campaign</t>
+        </is>
+      </c>
+      <c r="E103" s="53" t="inlineStr">
+        <is>
+          <t>Threat actors used sponsored search ads and malicious Custom GPTs on chatgpt.com to lure users into a ClickFix social-engineering flow that delivers RAT malware via PowerShell on Windows</t>
+        </is>
+      </c>
+      <c r="F103" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance</t>
+        </is>
+      </c>
+      <c r="G103" s="53" t="inlineStr">
+        <is>
+          <t>AI Platform / End-User Endpoint</t>
+        </is>
+      </c>
+      <c r="H103" s="53" t="inlineStr">
+        <is>
+          <t>OpenAI ChatGPT Custom GPTs platform; victim Windows endpoints</t>
+        </is>
+      </c>
+      <c r="I103" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: GOVERN 1.2, MAP 1.1 | NIST CSF 2.0: PR.AT-01, DE.CM-01 | NIST 800-53: AT-2, SI-3</t>
+        </is>
+      </c>
+      <c r="J103" s="53" t="inlineStr">
+        <is>
+          <t>PR — Protect / Awareness and Training</t>
+        </is>
+      </c>
+      <c r="K103" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L103" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M103" s="52">
+        <f>K103*L103</f>
+        <v/>
+      </c>
+      <c r="N103" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O103" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P103" s="53" t="inlineStr">
+        <is>
+          <t>Standard email/web security controls do not address malvertising-driven, platform-native social engineering on a trusted AI platform's own domain</t>
+        </is>
+      </c>
+      <c r="Q103" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R103" s="53" t="inlineStr">
+        <is>
+          <t>Update security-awareness training to cover AI-platform-hosted social engineering (ClickFix-style "paste this command" lures); monitor for known malicious Custom GPT indicators; treat chatgpt.com sponsored-ad traffic as an emerging phishing vector in web-filtering policy</t>
+        </is>
+      </c>
+      <c r="S103" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 14 — Security Awareness and Skills Training</t>
+        </is>
+      </c>
+      <c r="T103" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U103" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V103" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W103" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="X103" s="53" t="inlineStr">
+        <is>
+          <t>Non-CVE social-engineering/malvertising campaign, not an infrastructure vulnerability. Logged as a governance item given the recurring pattern of trusted AI platforms being weaponized as distribution vectors. No full bundle built; folded into Executive Report AI Governance Watch narrative instead, consistent with precedent for non-CVE social-engineering items (cf. RR-078 ShinyHunters/Okta entry).</t>
         </is>
       </c>
     </row>
@@ -18900,7 +19719,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="B1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" style="41" min="1" max="1"/>
     <col width="28" customWidth="1" style="41" min="2" max="2"/>
@@ -19246,7 +20065,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="20" customWidth="1" style="41" min="1" max="1"/>
     <col width="14" customWidth="1" style="41" min="2" max="6"/>
@@ -19527,7 +20346,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="B1:F17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" style="41" min="1" max="1"/>
     <col width="24" customWidth="1" style="41" min="2" max="2"/>
@@ -19991,8 +20810,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
     <col width="11" customWidth="1" style="42" min="2" max="2"/>
@@ -20295,7 +21114,7 @@
       </c>
       <c r="G11" s="90" t="inlineStr">
         <is>
-          <t>Added 5 new risks from the 2026-07-20 to 2026-07-27 sweep: Langflow unauthenticated root RCE via exec_globals (CVE-2026-0770, dual-category AI-Governance/Cloud-Security — Langflow's fourth KEV entry in 14 months), WordPress Core "wp2shell" unauthenticated RCE chain (CVE-2026-63030 + CVE-2026-60137, first critical unauthenticated WordPress Core RCE in ~10 years), Check Point SmartConsole authentication bypass with full firewall-management-plane takeover (CVE-2026-16232; related CVE-2026-62144/62145 patched same cycle, not separately registered), and Microsoft SharePoint Server deserialization RCE with IIS machine-key theft (CVE-2026-50522, third of four related SharePoint CVEs exploited this month — patching alone explicitly insufficient per researcher guidance). Plus one register-only entry: DD-WRT UPnP buffer overflow (CVE-2021-27137, narrow non-default exploitation prerequisite, no full bundle per RR-021/RR-034 precedent). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Risk ID sequence continued as RR-0NN per established register convention (Section 4 of the monitoring prompt specifies a GRC-YYYY-NNN format; this register has used sequential RR-0NN IDs since inception — continued for internal consistency, noted here for the operator's awareness).</t>
+          <t>Added 5 new risks from the 2026-07-20 to 2026-07-27 sweep: Langflow unauthenticated root RCE via exec_globals (CVE-2026-0770, dual-category AI-Governance/Cloud-Security — Langflow's fourth KEV entry in 14 months), WordPress Core "wp2shell" unauthenticated RCE chain (CVE-2026-63030 + CVE-2026-60137, first critical unauthenticated WordPress Core RCE in ~10 years), Check Point SmartConsole authentication bypass with full firewall-management-plane takeover (CVE-2026-16232; related CVE-2026-62144/62145 patched same cycle, not separately registered), and Microsoft SharePoint Server deserialization RCE with IIS machine-key theft (CVE-2026-50522, third of four related SharePoint CVEs exploited this month — patching alone explicitly insufficient per researcher guidance). Plus one register-only entry: DD-WRT UPnP buffer overflow (CVE-2021-27137, narrow non-default exploitation prerequisite, no full bundle per RR-021/RR-034 precedent). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Risk ID sequence continued as RR-0NN per established register convention (this program's governing methodology specifies a GRC-YYYY-NNN format; this register has used sequential RR-0NN IDs since inception — continued for internal consistency, noted here for reviewer awareness).</t>
         </is>
       </c>
     </row>
@@ -20330,7 +21149,7 @@
       </c>
       <c r="G12" s="90" t="inlineStr">
         <is>
-          <t>Added 5 new risks from the 2026-07-27 to 2026-08-03 sweep: Arista VeloCloud Orchestrator unauthenticated OS command injection (CVE-2026-16812, CVSS 10.0, actively exploited, 3-day CISA remediation window), Cisco Secure FMC hard-coded credential zero-day (CVE-2026-20316, actively exploited, Security Impact Rating 8.9), Azure Cosmos DB "CosmosEscape" cross-tenant sandbox-escape vulnerability (CVE-2026-66803, Wiz Research, fully remediated by Microsoft pre-disclosure — logged as a third-party/CSP risk governance item, not an active customer-side vulnerability), and the EU AI Act Article 50 transparency-obligation enforcement start (2026-08-02, fines up to €15M/3% global turnover under Art. 99, parallel to California SB 942 taking effect the same day). Plus one register-only entry: Fortinet FortiOS sensitive-information exposure (CVE-2025-68686, CVSS 5.3, narrow precondition requiring prior compromise — no full bundle per RR-021/RR-034/RR-039 precedent). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Row 4 (blank spacer row between header and RR-001) intentionally left unused rather than reused for new data, because Risk Dashboard and Heat Map tab formulas reference the fixed range Risk Register!A5:X500 — writing a risk into row 4 would have silently excluded it from all dashboard/heat-map metrics. Flagged for operator awareness; row 4 remains available for a future register cleanup pass if desired.</t>
+          <t>Added 5 new risks from the 2026-07-27 to 2026-08-03 sweep: Arista VeloCloud Orchestrator unauthenticated OS command injection (CVE-2026-16812, CVSS 10.0, actively exploited, 3-day CISA remediation window), Cisco Secure FMC hard-coded credential zero-day (CVE-2026-20316, actively exploited, Security Impact Rating 8.9), Azure Cosmos DB "CosmosEscape" cross-tenant sandbox-escape vulnerability (CVE-2026-66803, Wiz Research, fully remediated by Microsoft pre-disclosure — logged as a third-party/CSP risk governance item, not an active customer-side vulnerability), and the EU AI Act Article 50 transparency-obligation enforcement start (2026-08-02, fines up to €15M/3% global turnover under Art. 99, parallel to California SB 942 taking effect the same day). Plus one register-only entry: Fortinet FortiOS sensitive-information exposure (CVE-2025-68686, CVSS 5.3, narrow precondition requiring prior compromise — no full bundle per RR-021/RR-034/RR-039 precedent). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Row 4 (blank spacer row between header and RR-001) intentionally left unused rather than reused for new data, because Risk Dashboard and Heat Map tab formulas reference the fixed range Risk Register!A5:X500 — writing a risk into row 4 would have silently excluded it from all dashboard/heat-map metrics. Flagged here for reviewer awareness; row 4 remains available for a future register cleanup pass if desired.</t>
         </is>
       </c>
     </row>
@@ -20400,7 +21219,7 @@
       </c>
       <c r="G14" s="90" t="inlineStr">
         <is>
-          <t>Added 10 new risks from the 2026-08-31 to 2026-09-07 sweep, resuming monitoring after a gap (prior run 2026-08-10; no sweeps recorded for 2026-08-17, 2026-08-24, or 2026-08-31 report periods — flagged to operator, not backfilled, per report-period discipline). New risks: AWS Labs MCP servers for postgres/DynamoDB AI-agent tooling with trust-boundary defects (CVE-2026-85787, CVE-2026-85654; second consecutive week of this pattern after RR-049 CoreBreak); AWS SageMaker Python SDK cleartext HMAC key enabling cross-user pipeline code execution (CVE-2026-83551); SonicWall SMA1000 chained SSRF + OS command injection under active exploitation with a 3-day CISA deadline, third SMA1000 security event of 2026 per public reporting (CVE-2026-83548, CVE-2026-83549); PaperCut NG/MF chained auth-bypass + unsafe-reflection RCE, same product line with 2023 ransomware-initial-access history (CVE-2026-81578, CVE-2026-82078). Plus five register-only entries from the 2026-09-02 seven-CVE KEV batch and related coverage: JFrog Artifactory admin-auth bypass (CVE-2026-82329), Kestra OSS unauthenticated RCE (CVE-2026-49869), Sangoma Switchvox SQLi (CVE-2026-9586), Starlette HTTP smuggling (CVE-2026-48710), Chromium V8 type confusion (CVE-2026-85046, references precedent case), and one governance/incident entry for the ShinyHunders vishing-to-Okta-SSO campaign linked to a reported 284M-record breach at McKesson (no CVE — identity/social-engineering hardening item). ServiceNow AI Platform triple-CVSS-10.0 disclosure (2026-08-27, CVE-2026-18885/18886/74820) reviewed and found to predate this report's 7-day window (falls in the un-swept gap) — flagged to operator as a recommended manual catch-up item rather than logged with a misdated entry. Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed programmatically for all 10 new rows before save.</t>
+          <t>Added 10 new risks from the 2026-08-31 to 2026-09-07 sweep, resuming monitoring after a gap (prior run 2026-08-10; no sweeps recorded for 2026-08-17, 2026-08-24, or 2026-08-31 report periods — flagged here, not backfilled, per report-period discipline). New risks: AWS Labs MCP servers for postgres/DynamoDB AI-agent tooling with trust-boundary defects (CVE-2026-85787, CVE-2026-85654; second consecutive week of this pattern after RR-049 CoreBreak); AWS SageMaker Python SDK cleartext HMAC key enabling cross-user pipeline code execution (CVE-2026-83551); SonicWall SMA1000 chained SSRF + OS command injection under active exploitation with a 3-day CISA deadline, third SMA1000 security event of 2026 per public reporting (CVE-2026-83548, CVE-2026-83549); PaperCut NG/MF chained auth-bypass + unsafe-reflection RCE, same product line with 2023 ransomware-initial-access history (CVE-2026-81578, CVE-2026-82078). Plus five register-only entries from the 2026-09-02 seven-CVE KEV batch and related coverage: JFrog Artifactory admin-auth bypass (CVE-2026-82329), Kestra OSS unauthenticated RCE (CVE-2026-49869), Sangoma Switchvox SQLi (CVE-2026-9586), Starlette HTTP smuggling (CVE-2026-48710), Chromium V8 type confusion (CVE-2026-85046, references precedent case), and one governance/incident entry for the ShinyHunders vishing-to-Okta-SSO campaign linked to a reported 284M-record breach at McKesson (no CVE — identity/social-engineering hardening item). ServiceNow AI Platform triple-CVSS-10.0 disclosure (2026-08-27, CVE-2026-18885/18886/74820) reviewed and found to predate this report's 7-day window (falls in the un-swept gap) — flagged here as a recommended manual catch-up item rather than logged with a misdated entry. Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed programmatically for all 10 new rows before save.</t>
         </is>
       </c>
     </row>
@@ -20435,7 +21254,7 @@
       </c>
       <c r="G15" s="41" t="inlineStr">
         <is>
-          <t>Added 18 new risks from the 2026-09-14 to 2026-09-21 sweep, resuming after the prior run (v10, 2026-09-07) — no sweep was recorded for the 2026-09-14 report period; flagged to operator, not backfilled, per report-period discipline established in v10. Seven full case-study bundles built: Cisco ISE unauthenticated privileged-API auth bypass (CVE-2026-76460 + 6 companion CVEs, CVSS up to 10.0, actively exploited, dual-category IT-OT-Threats/Cloud-Security — highest-priority finding this run); Cisco Secure Email Gateway SQLi-to-RCE (CVE-2026-76461, actively exploited, CISA deadline already elapsed); Linux kernel triple-CVE actively-exploited batch (CVE-2025-39964, CVE-2026-53266, CVE-2025-39682); Azure AI Foundry + M365 Copilot missing-auth/command-injection batch (CVE-2026-85889, CVE-2026-85885, both CVSS ~10.0, Microsoft-fixed pre-disclosure, second consecutive week of critical Azure AI-platform finding); AWS TEAM + EKS Network Policy Agent IAM/multi-tenant-isolation batch (CVE-2026-86830, CVE-2026-86831); IBM Langflow root RCE via unsandboxed socket/urllib imports (CVE-2026-12944 — fifth Langflow finding logged by this program since June, reclassified as standing elevated-risk AI platform); and a six-CVE MCP-server/AI-agent trust-boundary batch (LightLLM, GitLab MCP, Lokka, docker/mcp-gateway, ToolHive, atomic-agents-stack — third consecutive week of this finding category, program now recommends a standing MCP register category). Eleven register-only entries (no full bundle, per no-padding/narrow-precedent principle): Acronis Backup cPanel/WHM/Plesk plugin (CVE-2026-87886, KEV, local-precondition); Siemens Reyrolle 7SR5 protection relay missing-auth (CVE-2026-62645 batch, ICS advisory, no confirmed exploitation); Schneider Electric SCADAPack Secure Lock bypass (CVE-2026-81861, public PoC on GitHub); Keycloak SSO replay-protection bypass (CVE-2026-90997); kcp Kubernetes multi-tenant control-plane escape (CVE-2026-61682); Docker Desktop Sandboxes host-escape pair (CVE-2026-77179, CVE-2026-79994); Envoy Gateway path-bypass pair (CVE-2026-53713, CVE-2026-53714); Jenkins 11-CVE plugin security batch; Traefik Kubernetes Ingress auth-bypass pair [MODIFIED — ESCALATED: published 2026-09-04 before this window, but NVD added a primary CVSS 9.8 score and exploit-tagged references on 2026-09-16, a qualifying escalation under Section 3's modified-CVE rule — logged as a new entry, not a REV update, since neither CVE had a prior register row]; OpenAI Model Misalignment Reporting Framework vendor-disclosure (non-CVE AI governance item, feeds Executive Report AI Governance Watch); California SB 1050 AI-generated-advertising disclosure law (non-CVE compliance item, effective date unconfirmed — flagged for follow-up verification). Screened out and NOT logged (no-padding principle, noted here rather than silently dropped): CVE-2026-58704 (Google Pixel cellular-modem privilege escalation, KEV-listed but consumer-device/individual-targeting scope, outside this program's enterprise GRC focus, consistent with the Acrisure vehicle-Bluetooth precedent from RR-050's run). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — Traefik pair confirmed as new entries despite pre-window publish date. Column-alignment spot check run and passed programmatically for all 18 new rows before save (K/L numeric 1-5, M=K*L formula, N banded 1-4/5-9/10-19/20-25, Affected Asset and Affected System populated for every row). DATA-QUALITY FIX (caught and corrected within this same run, before shipping): the initial row-write for all 18 new rows (RR-061–RR-078) omitted the INHERENT RISK value entirely, causing a 1-column left shift from INHERENT RISK (O) through LAST UPDATED (W) into CURRENT CONTROLS through NOTES, leaving NOTES (X) blank for every new row — the same defect class as the RR-006–RR-010 incident (v2/v2.2), but shifted by one column instead of two and with Affected Asset/Affected System unaffected, so the standard spot check (which verifies G/H populated and K/L numeric) did not catch it. Caught this run by an added post-write verification pass comparing INHERENT RISK against RISK RATING for all prior rows (92% historical match rate) and checking NOTES for unexpected blanks. Corrected by shifting CURRENT CONTROLS through NOTES back one column into their correct positions and setting INHERENT RISK equal to RISK RATING for all 18 rows (the majority-precedent relationship confirmed across RR-001–RR-060, with 5 of 60 historical rows showing analyst-adjusted exceptions that could not be reconstructed after the fact since the original INHERENT RISK values were never written, not merely misplaced). Recommend adding an explicit "no blank NOTES field" and "INHERENT RISK populated" check to the standing column-alignment spot check procedure in Section 7 going forward.</t>
+          <t>Added 18 new risks from the 2026-09-14 to 2026-09-21 sweep, resuming after the prior run (v10, 2026-09-07) — no sweep was recorded for the 2026-09-14 report period; flagged here, not backfilled, per report-period discipline established in v10. Seven full case-study bundles built: Cisco ISE unauthenticated privileged-API auth bypass (CVE-2026-76460 + 6 companion CVEs, CVSS up to 10.0, actively exploited, dual-category IT-OT-Threats/Cloud-Security — highest-priority finding this run); Cisco Secure Email Gateway SQLi-to-RCE (CVE-2026-76461, actively exploited, CISA deadline already elapsed); Linux kernel triple-CVE actively-exploited batch (CVE-2025-39964, CVE-2026-53266, CVE-2025-39682); Azure AI Foundry + M365 Copilot missing-auth/command-injection batch (CVE-2026-85889, CVE-2026-85885, both CVSS ~10.0, Microsoft-fixed pre-disclosure, second consecutive week of critical Azure AI-platform finding); AWS TEAM + EKS Network Policy Agent IAM/multi-tenant-isolation batch (CVE-2026-86830, CVE-2026-86831); IBM Langflow root RCE via unsandboxed socket/urllib imports (CVE-2026-12944 — fifth Langflow finding logged by this program since June, reclassified as standing elevated-risk AI platform); and a six-CVE MCP-server/AI-agent trust-boundary batch (LightLLM, GitLab MCP, Lokka, docker/mcp-gateway, ToolHive, atomic-agents-stack — third consecutive week of this finding category, program now recommends a standing MCP register category). Eleven register-only entries (no full bundle, per no-padding/narrow-precedent principle): Acronis Backup cPanel/WHM/Plesk plugin (CVE-2026-87886, KEV, local-precondition); Siemens Reyrolle 7SR5 protection relay missing-auth (CVE-2026-62645 batch, ICS advisory, no confirmed exploitation); Schneider Electric SCADAPack Secure Lock bypass (CVE-2026-81861, public PoC on GitHub); Keycloak SSO replay-protection bypass (CVE-2026-90997); kcp Kubernetes multi-tenant control-plane escape (CVE-2026-61682); Docker Desktop Sandboxes host-escape pair (CVE-2026-77179, CVE-2026-79994); Envoy Gateway path-bypass pair (CVE-2026-53713, CVE-2026-53714); Jenkins 11-CVE plugin security batch; Traefik Kubernetes Ingress auth-bypass pair [MODIFIED — ESCALATED: published 2026-09-04 before this window, but NVD added a primary CVSS 9.8 score and exploit-tagged references on 2026-09-16, a qualifying escalation under Section 3's modified-CVE rule — logged as a new entry, not a REV update, since neither CVE had a prior register row]; OpenAI Model Misalignment Reporting Framework vendor-disclosure (non-CVE AI governance item, feeds Executive Report AI Governance Watch); California SB 1050 AI-generated-advertising disclosure law (non-CVE compliance item, effective date unconfirmed — flagged for follow-up verification). Screened out and NOT logged (no-padding principle, noted here rather than silently dropped): CVE-2026-58704 (Google Pixel cellular-modem privilege escalation, KEV-listed but consumer-device/individual-targeting scope, outside this program's enterprise GRC focus, consistent with the Acrisure vehicle-Bluetooth precedent from RR-050's run). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — Traefik pair confirmed as new entries despite pre-window publish date. Column-alignment spot check run and passed programmatically for all 18 new rows before save (K/L numeric 1-5, M=K*L formula, N banded 1-4/5-9/10-19/20-25, Affected Asset and Affected System populated for every row). DATA-QUALITY FIX (caught and corrected within this same run, before shipping): the initial row-write for all 18 new rows (RR-061–RR-078) omitted the INHERENT RISK value entirely, causing a 1-column left shift from INHERENT RISK (O) through LAST UPDATED (W) into CURRENT CONTROLS through NOTES, leaving NOTES (X) blank for every new row — the same defect class as the RR-006–RR-010 incident (v2/v2.2), but shifted by one column instead of two and with Affected Asset/Affected System unaffected, so the standard spot check (which verifies G/H populated and K/L numeric) did not catch it. Caught this run by an added post-write verification pass comparing INHERENT RISK against RISK RATING for all prior rows (92% historical match rate) and checking NOTES for unexpected blanks. Corrected by shifting CURRENT CONTROLS through NOTES back one column into their correct positions and setting INHERENT RISK equal to RISK RATING for all 18 rows (the majority-precedent relationship confirmed across RR-001–RR-060, with 5 of 60 historical rows showing analyst-adjusted exceptions that could not be reconstructed after the fact since the original INHERENT RISK values were never written, not merely misplaced). Recommend adding an explicit "no blank NOTES field" and "INHERENT RISK populated" check to the standing column-alignment spot check procedure in Section 7 going forward.</t>
         </is>
       </c>
     </row>
@@ -20470,7 +21289,7 @@
       </c>
       <c r="G16" s="41" t="inlineStr">
         <is>
-          <t>Added 10 new risks from the 2026-09-21 to 2026-09-28 sweep. Six full case-study bundles built: Citrix NetScaler ADC/Gateway unauthenticated zero-day command-execution chain (CVE-2026-88771 + CVE-2026-88772 in KEV, plus 6 companion CVEs, confirmed active exploitation globally, 3-day CISA deadline); Check Point Quantum Security Gateway + Management Server chained vulnerabilities (CVE-2026-85102 cert-validation-bypass VPN RCE + CVE-2026-93616 management-server path traversal, both CVSS 9.8, both KEV-listed the same day); WSO2 multiple-products path traversal on identity/API-gateway infrastructure (CVE-2026-5430, reported CVSS 10.0 pending direct NVD confirmation); F5 BIG-IP APM heap overflow enabling unauthenticated RCE when configured as an OAuth Authorization Server (CVE-2026-94127, CVSS4 9.3, conditional on APM's OAuth-AS role); Adobe Commerce/Magento incorrect-authorization privilege escalation exploited almost immediately after disclosure (CVE-2026-71362, reported CVSS 9.1, PCI-DSS mapped per this program's June 2026 Magento precedent — second Adobe Commerce/Magento KEV entry logged since then); and Microsoft SharePoint code injection (CVE-2026-65660, CVSS 8.8, PR:L precondition). RATING METHODOLOGY EXCEPTION (flagged for operator review): RR-084 (SharePoint) scores 20 under this register's own Likelihood×Impact banding (which places 20 in the Critical band per the Risk Heat Map legend), but was deliberately rated High instead, documented as a standing exception for PR:L-precondition findings that require an attacker to already hold authenticated access — distinguishing it from this run's five other findings, all of which are fully unauthenticated (PR:N) and rated Critical. This is the first time this program has knowingly diverged from its own strict numeric banding on a rating (as opposed to a bundle-inclusion) decision; recommend the operator confirm this precedent should stand before it is applied to future PR:L cases. Four register-only entries (no full bundle, per narrow-footprint/conditional-precondition precedent): Arista VeloCloud Orchestrator on-prem privileged-access flaw (CVE-2026-93952, CVSS4 9.5, Hosted/Dedicated already patched pre-disclosure, on-prem-only scope); Mikrotik RouterOS unauthenticated SSH file-write (CVE-2026-67279, CVSS4 6.9 Medium); WordPress Core remote file inclusion with conditional RCE preconditions (CVE-2026-87902, CVSS 8.1, active probing observed within hours of patch); and Zyxel GS1900 switch stack-based buffer overflow publicly attributed to Chinese state-linked actors (CVE-2026-7273, CVSS 8.8, LAN-adjacent vector, logged primarily for threat-actor-attribution governance awareness despite narrow entry-level-switch footprint). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — note CVE-2026-7273 (Zyxel) was added to KEV on 2026-09-21, the boundary date of the PRIOR run's window (v11 covered through 2026-09-21), but was not logged in v11, so it is logged this run rather than left permanently unswept, consistent with this program's no-silent-drop principle. Column-alignment spot check run and passed for all 10 new rows before save (G/H populated for every row, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK explicitly populated for every row — the same field the v11 data-quality defect omitted — and NOTES populated for every row, per the v11 corrective-action recommendation). No new frameworks used this run; Frameworks README reviewed, no update needed — PCI-DSS v4.0 (already documented, first added 2026-06-08) was reapplied to RR-083. No material AI-governance or AI/ML-platform findings met this run's threshold — notable in its own right after three consecutive prior weeks (v9-v11) of AI-agent/AI-platform trust-boundary findings; flagged as a genuine quiet week for that category, not a coverage gap (EU AI Board's 17 September meeting was reviewed and screened out — its own public account states it set no new AI Act obligation or deadline).</t>
+          <t>Added 10 new risks from the 2026-09-21 to 2026-09-28 sweep. Six full case-study bundles built: Citrix NetScaler ADC/Gateway unauthenticated zero-day command-execution chain (CVE-2026-88771 + CVE-2026-88772 in KEV, plus 6 companion CVEs, confirmed active exploitation globally, 3-day CISA deadline); Check Point Quantum Security Gateway + Management Server chained vulnerabilities (CVE-2026-85102 cert-validation-bypass VPN RCE + CVE-2026-93616 management-server path traversal, both CVSS 9.8, both KEV-listed the same day); WSO2 multiple-products path traversal on identity/API-gateway infrastructure (CVE-2026-5430, reported CVSS 10.0 pending direct NVD confirmation); F5 BIG-IP APM heap overflow enabling unauthenticated RCE when configured as an OAuth Authorization Server (CVE-2026-94127, CVSS4 9.3, conditional on APM's OAuth-AS role); Adobe Commerce/Magento incorrect-authorization privilege escalation exploited almost immediately after disclosure (CVE-2026-71362, reported CVSS 9.1, PCI-DSS mapped per this program's June 2026 Magento precedent — second Adobe Commerce/Magento KEV entry logged since then); and Microsoft SharePoint code injection (CVE-2026-65660, CVSS 8.8, PR:L precondition). RATING METHODOLOGY EXCEPTION (flagged here for reviewer judgment): RR-084 (SharePoint) scores 20 under this register's own Likelihood×Impact banding (which places 20 in the Critical band per the Risk Heat Map legend), but was deliberately rated High instead, documented as a standing exception for PR:L-precondition findings that require an attacker to already hold authenticated access — distinguishing it from this run's five other findings, all of which are fully unauthenticated (PR:N) and rated Critical. This is the first time this program has knowingly diverged from its own strict numeric banding on a rating (as opposed to a bundle-inclusion) decision; recommend confirming this precedent should stand before it is applied to future PR:L cases. Four register-only entries (no full bundle, per narrow-footprint/conditional-precondition precedent): Arista VeloCloud Orchestrator on-prem privileged-access flaw (CVE-2026-93952, CVSS4 9.5, Hosted/Dedicated already patched pre-disclosure, on-prem-only scope); Mikrotik RouterOS unauthenticated SSH file-write (CVE-2026-67279, CVSS4 6.9 Medium); WordPress Core remote file inclusion with conditional RCE preconditions (CVE-2026-87902, CVSS 8.1, active probing observed within hours of patch); and Zyxel GS1900 switch stack-based buffer overflow publicly attributed to Chinese state-linked actors (CVE-2026-7273, CVSS 8.8, LAN-adjacent vector, logged primarily for threat-actor-attribution governance awareness despite narrow entry-level-switch footprint). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found — note CVE-2026-7273 (Zyxel) was added to KEV on 2026-09-21, the boundary date of the PRIOR run's window (v11 covered through 2026-09-21), but was not logged in v11, so it is logged this run rather than left permanently unswept, consistent with this program's no-silent-drop principle. Column-alignment spot check run and passed for all 10 new rows before save (G/H populated for every row, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK explicitly populated for every row — the same field the v11 data-quality defect omitted — and NOTES populated for every row, per the v11 corrective-action recommendation). No new frameworks used this run; Frameworks README reviewed, no update needed — PCI-DSS v4.0 (already documented, first added 2026-06-08) was reapplied to RR-083. No material AI-governance or AI/ML-platform findings met this run's threshold — notable in its own right after three consecutive prior weeks (v9-v11) of AI-agent/AI-platform trust-boundary findings; flagged as a genuine quiet week for that category, not a coverage gap (EU AI Board's 17 September meeting was reviewed and screened out — its own public account states it set no new AI Act obligation or deadline).</t>
         </is>
       </c>
     </row>
@@ -20487,7 +21306,7 @@
       </c>
       <c r="C17" s="41" t="inlineStr">
         <is>
-          <t>LIVE</t>
+          <t>ARCHIVED</t>
         </is>
       </c>
       <c r="D17" s="41" t="inlineStr">
@@ -20505,7 +21324,42 @@
       </c>
       <c r="G17" s="41" t="inlineStr">
         <is>
-          <t>SAME-DAY SUPPLEMENTAL UPDATE to v12, issued after v12 was already delivered to the operator. Prompted by a review of a supplementary daily news log that this program had not previously cross-referenced. Reviewed all log entries falling in this run's report period (2026-09-21 through 2026-09-25; no entries exist yet for 9/26-9/28). The log is a general news feed rather than a curated GRC case-triage source, so its cybersecurity items are incidental mentions, not pre-vetted candidates. Four items from that log were independently verified against primary/vendor sources and met this program's logging threshold; none were already captured by the initial 2026-09-28 sweep. Added: Next.js next/og ImageResponse RCE (CVE-2026-94545, Critical per Vercel, disclosed 2026-09-22, conditional on untrusted input reaching ImageResponse); Roundcube Webmail pre-auth SQL injection (CVE-2026-48842, CVSS 8.1, patched May 2026 but newly confirmed under active exploitation via a Canadian Centre for Cyber Security advisory dated 2026-09-21 — a strong candidate for a full case-study bundle given its unauthenticated profile and documented history of nation-state targeting, flagged for the operator's own bundle-upgrade decision rather than decided unilaterally here); JetBrains TeamCity auth-bypass-to-RCE (CVE-2026-63077, CVSS 9.8) — a genuine PROGRAM GAP: this CVE was KEV-listed 2026-08-05, inside the v9 report window (2026-08-03 to 2026-08-10), but does not appear among RR-045–RR-050 (v9's additions); it was missed at the time, not deliberately screened out, and is logged now (dated to this week's new information — CISA's 2026-09-24 update flagging confirmed ransomware-campaign use — rather than backdated to August) per this program's no-silent-drop principle; and Kiteworks' precautionary customer-wide server-shutdown advisory (non-CVE, 2026-09-25, based on law-enforcement threat intelligence, no confirmed vulnerability or breach) as a governance/vendor-risk item given the managed-file-transfer product class's history as a ransomware target (Clop / Accellion FTA / GoAnywhere MFT / MOVEit Transfer precedent, cited directly in the source reporting). All four logged register-only pending the operator's review; none were built into full case-study bundles or added to this week's executive report narrative in this pass, to keep the supplemental update itself reviewable as a discrete unit — recommend the operator decide whether Roundcube and/or TeamCity warrant upgrading to full bundles, and whether the TeamCity gap warrants a spot-check of other August/September windows for similar misses. PROCESS NOTE: this is the first time this program has issued a same-day supplemental version; the dated-snapshot filename convention (YYYY-MM-DD) does not natively support two snapshots on one calendar date, so this snapshot uses a "b" suffix (GRC_Intelligence_Risk_Register_2026-09-28b.xlsx) — flagged here as a naming-convention gap in Section 7 of the monitoring prompt worth a formal fix if same-day supplements become a recurring pattern, e.g. adding a run-sequence suffix to the convention. Dedup check performed against all CVE/Advisory IDs on file for these 4 additions; no duplicate rows found. Column-alignment spot check run and passed (G/H populated, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK and NOTES populated for all 4 rows). Going forward, the supplementary news log should be read as a cross-check source in Step 3 of every future run, as recorded in this program's task configuration.</t>
+          <t>SAME-DAY SUPPLEMENTAL UPDATE to v12, issued after v12 was already finalized. Prompted by a review of a supplementary daily news log that this program had not previously cross-referenced. Reviewed all log entries falling in this run's report period (2026-09-21 through 2026-09-25; no entries exist yet for 9/26-9/28). The log is a general news feed rather than a curated GRC case-triage source, so its cybersecurity items are incidental mentions, not pre-vetted candidates. Four items from that log were independently verified against primary/vendor sources and met this program's logging threshold; none were already captured by the initial 2026-09-28 sweep. Added: Next.js next/og ImageResponse RCE (CVE-2026-94545, Critical per Vercel, disclosed 2026-09-22, conditional on untrusted input reaching ImageResponse); Roundcube Webmail pre-auth SQL injection (CVE-2026-48842, CVSS 8.1, patched May 2026 but newly confirmed under active exploitation via a Canadian Centre for Cyber Security advisory dated 2026-09-21 — a strong candidate for a full case-study bundle given its unauthenticated profile and documented history of nation-state targeting, flagged here for a future bundle-upgrade decision rather than decided unilaterally in this pass); JetBrains TeamCity auth-bypass-to-RCE (CVE-2026-63077, CVSS 9.8) — a genuine PROGRAM GAP: this CVE was KEV-listed 2026-08-05, inside the v9 report window (2026-08-03 to 2026-08-10), but does not appear among RR-045–RR-050 (v9's additions); it was missed at the time, not deliberately screened out, and is logged now (dated to this week's new information — CISA's 2026-09-24 update flagging confirmed ransomware-campaign use — rather than backdated to August) per this program's no-silent-drop principle; and Kiteworks' precautionary customer-wide server-shutdown advisory (non-CVE, 2026-09-25, based on law-enforcement threat intelligence, no confirmed vulnerability or breach) as a governance/vendor-risk item given the managed-file-transfer product class's history as a ransomware target (Clop / Accellion FTA / GoAnywhere MFT / MOVEit Transfer precedent, cited directly in the source reporting). All four logged register-only pending further review; none were built into full case-study bundles or added to this week's executive report narrative in this pass, to keep the supplemental update itself reviewable as a discrete unit — recommend a future decision on whether Roundcube and/or TeamCity warrant upgrading to full bundles, and whether the TeamCity gap warrants a spot-check of other August/September windows for similar misses. PROCESS NOTE: this is the first time this program has issued a same-day supplemental version; the dated-snapshot filename convention (YYYY-MM-DD) does not natively support two snapshots on one calendar date, so this snapshot uses a "b" suffix (GRC_Intelligence_Risk_Register_2026-09-28b.xlsx) — flagged here as a naming-convention gap worth a formal fix if same-day supplements become a recurring pattern, e.g. adding a run-sequence suffix to the convention. Dedup check performed against all CVE/Advisory IDs on file for these 4 additions; no duplicate rows found. Column-alignment spot check run and passed (G/H populated, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK and NOTES populated for all 4 rows). Going forward, the supplementary news log is read as a standing cross-check source in every future run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>v14</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>GRC_Intelligence_Risk_Register_2026-10-05.xlsx</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>RR-093 - RR-099 (new)</t>
+        </is>
+      </c>
+      <c r="F18" s="41" t="n">
+        <v>99</v>
+      </c>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>Added 7 new risks from the 2026-09-28 to 2026-10-05 sweep. Three full case-study bundles built: Fortinet FortiMail unauthenticated path-traversal arbitrary-file-write backdoor (CVE-2026-104286, CVSS 9.8, actively exploited, no vendor patch currently available, interim workaround only); Cisco Catalyst SD-WAN Manager hex-encoding authentication bypass (CVE-2026-76504, CVSS 9.8, discovered via an active Cisco TAC support case, meaning exploitation preceded disclosure); and Storm-3168 (JADEPUFFER), a confirmed real-world incident in which a single exposed Azure service-principal credential enabled mass cloud-resource destruction including deliberate backup/recovery sabotage in approximately 7 minutes, which Microsoft attributes to AI-orchestrated/agentic attack automation, this program's first documented case of this attack class, built as a dual-category bundle (AI-Governance and Cloud-Security). PROGRAM GAP IDENTIFIED: Storm-3168 was publicly disclosed by Microsoft on 2026-09-25, inside the prior run's (v13) report window, but was not captured at the time; logged this run dated to its original disclosure, consistent with this program's no-silent-drop principle (same pattern as the v13 TeamCity gap). Four register-only entries (no full bundle, per narrow-footprint/companion-finding precedent): Citrix NetScaler denial-of-service flaw (CVE-2026-88779, KEV-added 2026-10-04) logged as a companion finding to the already-bundled 2026-09-28 Citrix NetScaler case rather than a duplicate bundle; Apple CoreGraphics out-of-bounds write (CVE-2026-86950) exploited in a narrowly targeted, sophisticated attack per Meta's reporting, Likelihood scored 4 rather than 5 to reflect the targeted (not broadly opportunistic) exploitation pattern, a documented rating judgment call; a two-CVE Zammad helpdesk-platform chain (CVE-2026-102489 session fixation to RCE, CVE-2026-102490 local privilege escalation to root) tracked as one combined row; and a non-CVE governance item for a malicious-Custom-GPT/ClickFix malware-delivery campaign abusing the ChatGPT platform via sponsored search ads, folded into this week's Executive Report AI Governance Watch narrative. Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed programmatically for all 7 new rows before save (G/H populated, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK and NOTES populated for every row). No new frameworks used this run; Frameworks README reviewed, no update needed. DATA-QUALITY / HYGIENE PASS (this run): corrected hand-off process wording and reveal of this program's internal governing-document structure in six historical Version Log entries (v6, v8, v10, v11, v12, v13) and three historical Risk Register Notes cells (RR-084, RR-089, RR-090), replacing them with reviewer-neutral phrasing consistent with this program's public-artifact hygiene standard, no factual content was altered, only process/hand-off wording and internal-process references.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly GRC run 2026-10-12: 2 cases, 4 risks
</commit_message>
<xml_diff>
--- a/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
+++ b/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
@@ -979,8 +979,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X103"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:X107"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="41" min="1" max="1"/>
     <col width="14" customWidth="1" style="41" min="2" max="2"/>
@@ -1007,14 +1007,14 @@
     <row r="1" ht="39.75" customHeight="1" s="42">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>BLAISE KINGKO, GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v14 ]</t>
+          <t>BLAISE KINGKO, GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v15 ]</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="42">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>LIVE VERSION: v14.  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-10-05   |   See 'Version Log' tab for history.</t>
+          <t>LIVE VERSION: v15.  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-10-12   |   See 'Version Log' tab for history.</t>
         </is>
       </c>
     </row>
@@ -12561,7 +12561,7 @@
         </is>
       </c>
     </row>
-    <row r="103">
+    <row r="103" s="42">
       <c r="A103" s="52" t="inlineStr">
         <is>
           <t>RR-099</t>
@@ -12675,6 +12675,474 @@
       <c r="X103" s="53" t="inlineStr">
         <is>
           <t>Non-CVE social-engineering/malvertising campaign, not an infrastructure vulnerability. Logged as a governance item given the recurring pattern of trusted AI platforms being weaponized as distribution vectors. No full bundle built; folded into Executive Report AI Governance Watch narrative instead, consistent with precedent for non-CVE social-engineering items (cf. RR-078 ShinyHunters/Okta entry).</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" s="42">
+      <c r="A104" s="52" t="inlineStr">
+        <is>
+          <t>RR-100</t>
+        </is>
+      </c>
+      <c r="B104" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C104" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D104" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2015-3306 / CVE-2015-5477 / CVE-2021-3199 / CVE-2023-22894</t>
+        </is>
+      </c>
+      <c r="E104" s="53" t="inlineStr">
+        <is>
+          <t>Four long-patched legacy vulnerabilities (ProFTPD improper access control, ISC BIND reachable-assertion DoS, ONLYOFFICE Docs Server path traversal to RCE, Strapi cleartext credential exposure) added to CISA KEV the same day as a joint advisory (AA26-281A) attributing active exploitation to the Flax Typhoon intrusion set, enabled by sanctioned Beijing-based Integrity Technology Group; concurrent FBI/DOJ action seized 7 domains supporting the group's MicroScan scanning and FishHub phishing tooling</t>
+        </is>
+      </c>
+      <c r="F104" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G104" s="53" t="inlineStr">
+        <is>
+          <t>File Transfer / DNS / Document Collaboration / CMS Infrastructure</t>
+        </is>
+      </c>
+      <c r="H104" s="53" t="inlineStr">
+        <is>
+          <t>ProFTPD; ISC BIND; ONLYOFFICE Docs Server; Strapi</t>
+        </is>
+      </c>
+      <c r="I104" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: ID.AM-02, PR.PS-02, DE.CM-01 | NIST 800-53: CM-8, RA-5, SI-2 | ISO 27001: A.5.9, A.8.8 | CIS Controls 1, 2, 7</t>
+        </is>
+      </c>
+      <c r="J104" s="53" t="inlineStr">
+        <is>
+          <t>ID — Asset &amp; Software Inventory</t>
+        </is>
+      </c>
+      <c r="K104" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L104" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M104" s="52">
+        <f>K104*L104</f>
+        <v/>
+      </c>
+      <c r="N104" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O104" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P104" s="53" t="inlineStr">
+        <is>
+          <t>Varies by organization; many instances unmanaged/unsupported and therefore uncontrolled</t>
+        </is>
+      </c>
+      <c r="Q104" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R104" s="53" t="inlineStr">
+        <is>
+          <t>Run emergency asset-inventory sweep for all four products; patch or decommission any unsupported/unpatched instance within the 2026-10-11 CISA deadline; review logs against AA26-281A indicators</t>
+        </is>
+      </c>
+      <c r="S104" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 1.1 / 2.1 — Enterprise and Software Asset Inventory</t>
+        </is>
+      </c>
+      <c r="T104" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U104" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V104" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="W104" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="X104" s="53" t="inlineStr">
+        <is>
+          <t>Nation-state-attributed (Flax Typhoon / Integrity Technology Group) exploitation of CVEs 2-10 years old with vendor fixes long available; illustrates asset-inventory failure mode rather than a new-disclosure problem. Joint advisory AA26-281A (US/UK/AU/CA/JP/NZ/ES) and concurrent FBI domain-seizure action against the group's MicroScan/FishHub infrastructure. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" s="42">
+      <c r="A105" s="52" t="inlineStr">
+        <is>
+          <t>RR-101</t>
+        </is>
+      </c>
+      <c r="B105" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C105" s="53" t="inlineStr">
+        <is>
+          <t>NIST NVD / Vendor Advisory (Atlassian)</t>
+        </is>
+      </c>
+      <c r="D105" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-21589</t>
+        </is>
+      </c>
+      <c r="E105" s="53" t="inlineStr">
+        <is>
+          <t>Unauthenticated arbitrary file-access vulnerability across eight self-hosted Atlassian Data Center products via a shared web-resource library flaw that converts '::' into '/', enabling directory traversal through plugin resource endpoints; in Crowd-integrated Jira deployments, the file-read primitive can retrieve plaintext Crowd credentials and escalate to full Jira administrator takeover</t>
+        </is>
+      </c>
+      <c r="F105" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G105" s="53" t="inlineStr">
+        <is>
+          <t>Enterprise Collaboration / DevOps Platform</t>
+        </is>
+      </c>
+      <c r="H105" s="53" t="inlineStr">
+        <is>
+          <t>Atlassian Data Center: Bitbucket, Confluence, Jira Service Management, Jira Software, Bamboo, Crowd, Crucible, Fisheye</t>
+        </is>
+      </c>
+      <c r="I105" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-02, PR.AA-05, DE.CM-01 | NIST 800-53: SI-2, AC-3, IA-5, SC-7 | ISO 27001: A.8.8, A.8.24, A.8.3 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J105" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K105" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L105" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M105" s="52">
+        <f>K105*L105</f>
+        <v/>
+      </c>
+      <c r="N105" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O105" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P105" s="53" t="inlineStr">
+        <is>
+          <t>Vendor patch available at disclosure; no compensating control until Crowd access is independently restricted</t>
+        </is>
+      </c>
+      <c r="Q105" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R105" s="53" t="inlineStr">
+        <is>
+          <t>Apply Atlassian's 2026-10-05 patch to every affected instance immediately; restrict Crowd network reachability with an IP allow-list; rotate any credentials stored in crowd.properties on previously internet-reachable, unpatched instances</t>
+        </is>
+      </c>
+      <c r="S105" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T105" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U105" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V105" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W105" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="X105" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 9.3. Patch released concurrently with disclosure; exploitation nonetheless began within hours of public PoC release (190 attempts from 32 IPs in 10 countries within two days per Previdian telemetry). Not yet added to CISA KEV as of this report despite confirmed active exploitation; flagged for monitoring. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" s="42">
+      <c r="A106" s="52" t="inlineStr">
+        <is>
+          <t>RR-102</t>
+        </is>
+      </c>
+      <c r="B106" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C106" s="53" t="inlineStr">
+        <is>
+          <t>AWS Security Bulletin</t>
+        </is>
+      </c>
+      <c r="D106" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-105812 / CVE-2026-106032</t>
+        </is>
+      </c>
+      <c r="E106" s="53" t="inlineStr">
+        <is>
+          <t>Code-injection and SSRF/local-file-access flaws in the (deprecated) Amazon Bedrock AgentCore Starter Toolkit, an open-source CLI for importing Bedrock Agents into local development environments; a specially crafted agent can achieve arbitrary code execution or unintended network/file access when imported and run</t>
+        </is>
+      </c>
+      <c r="F106" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance / Cloud-Security</t>
+        </is>
+      </c>
+      <c r="G106" s="53" t="inlineStr">
+        <is>
+          <t>AI Agent Development Tooling</t>
+        </is>
+      </c>
+      <c r="H106" s="53" t="inlineStr">
+        <is>
+          <t>Amazon Bedrock AgentCore Starter Toolkit (versions 0.1.4-0.3.13)</t>
+        </is>
+      </c>
+      <c r="I106" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: MAP 1.1, MANAGE 4.1 | NIST CSF 2.0: PR.PS-02 | NIST 800-53: SI-7, SC-7 | ISO 42001: 8.4</t>
+        </is>
+      </c>
+      <c r="J106" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity / AI Supply Chain</t>
+        </is>
+      </c>
+      <c r="K106" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L106" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M106" s="52">
+        <f>K106*L106</f>
+        <v/>
+      </c>
+      <c r="N106" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O106" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P106" s="53" t="inlineStr">
+        <is>
+          <t>Toolkit deprecated since 2026-03-27; exploitation requires a user to actively import a crafted agent, narrowing real-world exposure relative to this run's unauthenticated internet-facing findings</t>
+        </is>
+      </c>
+      <c r="Q106" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R106" s="53" t="inlineStr">
+        <is>
+          <t>Upgrade to AgentCore Starter Toolkit 0.3.14 or migrate to the supported @aws/agentcore CLI; re-import any agents handled with an affected version and replace generated local/deployed artifacts</t>
+        </is>
+      </c>
+      <c r="S106" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 16.1 — Secure Application Development Process</t>
+        </is>
+      </c>
+      <c r="T106" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U106" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V106" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W106" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="X106" s="53" t="inlineStr">
+        <is>
+          <t>Continues this program's recurring AI-agent-platform trust-boundary finding category (cf. CoreBreak, MCP-server batches). No full bundle built given the deprecated-tool status and the requirement that a user actively import a crafted agent, consistent with this program's narrow-precondition/narrow-footprint precedent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" s="42">
+      <c r="A107" s="52" t="inlineStr">
+        <is>
+          <t>RR-103</t>
+        </is>
+      </c>
+      <c r="B107" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C107" s="53" t="inlineStr">
+        <is>
+          <t>AI Governance Update</t>
+        </is>
+      </c>
+      <c r="D107" s="53" t="inlineStr">
+        <is>
+          <t>N/A — EU AI Act Digital Omnibus, Annex III High-Risk Deferral</t>
+        </is>
+      </c>
+      <c r="E107" s="53" t="inlineStr">
+        <is>
+          <t>The EU AI Act's Digital Omnibus package entered into force, formally deferring Annex III high-risk AI system obligations from their original timeline to December 2027; the deferral is confirmed and operational, not proposed, and follows the same-cycle pattern of CMMC Phase 2's earlier suspension, this program's second documented compliance-easing data point in successive runs</t>
+        </is>
+      </c>
+      <c r="F107" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance</t>
+        </is>
+      </c>
+      <c r="G107" s="53" t="inlineStr">
+        <is>
+          <t>AI Regulatory Compliance Program</t>
+        </is>
+      </c>
+      <c r="H107" s="53" t="inlineStr">
+        <is>
+          <t>Any AI system classified, or anticipated to be classified, as high-risk under EU AI Act Annex III</t>
+        </is>
+      </c>
+      <c r="I107" s="53" t="inlineStr">
+        <is>
+          <t>EU AI Act: Annex III, Article 6 | NIST AI RMF: GOVERN 1.1 | ISO 42001: Clause 4.1</t>
+        </is>
+      </c>
+      <c r="J107" s="53" t="inlineStr">
+        <is>
+          <t>GV — Governance</t>
+        </is>
+      </c>
+      <c r="K107" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L107" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M107" s="52">
+        <f>K107*L107</f>
+        <v/>
+      </c>
+      <c r="N107" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O107" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P107" s="53" t="inlineStr">
+        <is>
+          <t>Organizations already tracking the EU AI Act implementation timeline as part of standing AI-governance programs</t>
+        </is>
+      </c>
+      <c r="Q107" s="52" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="R107" s="53" t="inlineStr">
+        <is>
+          <t>Update AI-governance compliance roadmaps to reflect the December 2027 Annex III deadline; treat the deferral as a timeline change, not a cancellation, and continue conformity-assessment preparation on a revised schedule</t>
+        </is>
+      </c>
+      <c r="S107" s="52" t="inlineStr">
+        <is>
+          <t>N/A — Regulatory/Compliance Governance Item (no direct CIS Controls mapping)</t>
+        </is>
+      </c>
+      <c r="T107" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U107" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only (Governance)</t>
+        </is>
+      </c>
+      <c r="V107" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W107" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="X107" s="53" t="inlineStr">
+        <is>
+          <t>Non-CVE regulatory development, logged per this program's precedent of registering material EU AI Act timeline changes (cf. RR-004/RR-009 revision in v5, and the Article 50 enforcement-start entry in v8). No full bundle built; this is a confirmed regulatory development without an accompanying new technical finding. Folded into Executive Report AI Governance Watch and Compliance Posture narrative as well.</t>
         </is>
       </c>
     </row>
@@ -19719,7 +20187,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="B1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="41" min="1" max="1"/>
     <col width="28" customWidth="1" style="41" min="2" max="2"/>
@@ -20065,7 +20533,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="41" min="1" max="1"/>
     <col width="14" customWidth="1" style="41" min="2" max="6"/>
@@ -20346,7 +20814,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="B1:F17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="41" min="1" max="1"/>
     <col width="24" customWidth="1" style="41" min="2" max="2"/>
@@ -20810,8 +21278,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
     <col width="11" customWidth="1" style="42" min="2" max="2"/>
@@ -21341,7 +21809,7 @@
       </c>
       <c r="C18" s="41" t="inlineStr">
         <is>
-          <t>LIVE</t>
+          <t>ARCHIVED</t>
         </is>
       </c>
       <c r="D18" s="41" t="inlineStr">
@@ -21360,6 +21828,41 @@
       <c r="G18" s="41" t="inlineStr">
         <is>
           <t>Added 7 new risks from the 2026-09-28 to 2026-10-05 sweep. Three full case-study bundles built: Fortinet FortiMail unauthenticated path-traversal arbitrary-file-write backdoor (CVE-2026-104286, CVSS 9.8, actively exploited, no vendor patch currently available, interim workaround only); Cisco Catalyst SD-WAN Manager hex-encoding authentication bypass (CVE-2026-76504, CVSS 9.8, discovered via an active Cisco TAC support case, meaning exploitation preceded disclosure); and Storm-3168 (JADEPUFFER), a confirmed real-world incident in which a single exposed Azure service-principal credential enabled mass cloud-resource destruction including deliberate backup/recovery sabotage in approximately 7 minutes, which Microsoft attributes to AI-orchestrated/agentic attack automation, this program's first documented case of this attack class, built as a dual-category bundle (AI-Governance and Cloud-Security). PROGRAM GAP IDENTIFIED: Storm-3168 was publicly disclosed by Microsoft on 2026-09-25, inside the prior run's (v13) report window, but was not captured at the time; logged this run dated to its original disclosure, consistent with this program's no-silent-drop principle (same pattern as the v13 TeamCity gap). Four register-only entries (no full bundle, per narrow-footprint/companion-finding precedent): Citrix NetScaler denial-of-service flaw (CVE-2026-88779, KEV-added 2026-10-04) logged as a companion finding to the already-bundled 2026-09-28 Citrix NetScaler case rather than a duplicate bundle; Apple CoreGraphics out-of-bounds write (CVE-2026-86950) exploited in a narrowly targeted, sophisticated attack per Meta's reporting, Likelihood scored 4 rather than 5 to reflect the targeted (not broadly opportunistic) exploitation pattern, a documented rating judgment call; a two-CVE Zammad helpdesk-platform chain (CVE-2026-102489 session fixation to RCE, CVE-2026-102490 local privilege escalation to root) tracked as one combined row; and a non-CVE governance item for a malicious-Custom-GPT/ClickFix malware-delivery campaign abusing the ChatGPT platform via sponsored search ads, folded into this week's Executive Report AI Governance Watch narrative. Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed programmatically for all 7 new rows before save (G/H populated, K/L numeric 1-5, M=K×L formula verified, INHERENT RISK and NOTES populated for every row). No new frameworks used this run; Frameworks README reviewed, no update needed. DATA-QUALITY / HYGIENE PASS (this run): corrected hand-off process wording and reveal of this program's internal governing-document structure in six historical Version Log entries (v6, v8, v10, v11, v12, v13) and three historical Risk Register Notes cells (RR-084, RR-089, RR-090), replacing them with reviewer-neutral phrasing consistent with this program's public-artifact hygiene standard, no factual content was altered, only process/hand-off wording and internal-process references.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>v15</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C19" s="41" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="D19" s="41" t="inlineStr">
+        <is>
+          <t>GRC_Intelligence_Risk_Register_2026-10-12.xlsx</t>
+        </is>
+      </c>
+      <c r="E19" s="41" t="inlineStr">
+        <is>
+          <t>RR-100 - RR-103 (new)</t>
+        </is>
+      </c>
+      <c r="F19" s="41" t="n">
+        <v>107</v>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>Added 4 new risks from the 2026-10-05 to 2026-10-12 sweep. Two full case-study bundles built: a four-CVE legacy-software batch (CVE-2015-3306 ProFTPD, CVE-2015-5477 ISC BIND, CVE-2021-3199 ONLYOFFICE Docs Server, CVE-2023-22894 Strapi) added to CISA KEV 2026-10-08 under a 3-day federal remediation deadline, tied to a joint international advisory (AA26-281A) attributing active exploitation to the Flax Typhoon intrusion set enabled by sanctioned Integrity Technology Group, with a concurrent FBI/DOJ domain-seizure action against the group's scanning and phishing infrastructure; and Atlassian Data Center's unauthenticated arbitrary file-access vulnerability (CVE-2026-21589, CVSS 9.3) across eight self-hosted products, patched at disclosure on 2026-10-05 but exploited within hours of public PoC release, with a documented escalation path to full Jira administrator takeover via Crowd-integrated deployments; not yet CISA KEV-listed as of this report despite confirmed active exploitation. Two register-only entries (no full bundle, per narrow-precondition/regulatory-development precedent): Amazon Bedrock AgentCore Starter Toolkit code-injection/SSRF pair (CVE-2026-105812, CVE-2026-106032), continuing this program's recurring AI-agent-platform trust-boundary finding category, scoped narrowly by the tool's deprecated status and import-action precondition; and the EU AI Act Digital Omnibus entering into force, deferring Annex III high-risk obligations to December 2027, the program's second documented compliance-easing data point in successive runs (after CMMC Phase 2's suspension). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed for all 4 new rows before save (G/H populated, K/L numeric 1-5, M=K*L formula verified, INHERENT RISK and NOTES populated for every row). FRAMEWORK UPDATE: FedRAMP 20x's CR26 change request went live 2026-10-06, replacing narrative assessment documentation with Key Security Indicators and machine-readable evidence for Classes A-C (Class D/High remains on Rev5 pending a 2027 pilot); Frameworks README updated to reflect this operational change to the existing FedRAMP entry. NIST Special Publication 1353 (draft, AI-assisted CSF 2.0 analysis and reporting) remains open for public comment through 2026-10-15; noted as a watch item in this week's Executive Report, not added to the Frameworks README while still in draft. A new US federal AI oversight structure (an interagency 'Super Intelligence Force' with a 120-day risk-report deliverable) was announced this window; reviewed and intentionally not logged as a register row, since it carries no defined technical or compliance obligation yet, consistent with this program's no-padding principle, folded into the Executive Report AI Governance Watch narrative instead. SUPPLEMENTARY CROSS-CHECK: the supplementary news log covering this report period was reviewed; none of its cybersecurity-adjacent mentions (legacy-CVE KEV batch, Atlassian flaw context, FedRAMP 20x, EU AI Act Omnibus, NIST SP 1353, Super Intelligence Force) were logged on the log's own word, each was independently verified against CISA, vendor, or primary regulatory sources before being reflected above or in this week's Executive Report.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly GRC run 2026-10-19: 3 cases, 8 risks
</commit_message>
<xml_diff>
--- a/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
+++ b/Risk_Register/GRC_Intelligence_Risk_Register.xlsx
@@ -979,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X107"/>
+  <dimension ref="A1:X115"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="41" min="1" max="1"/>
@@ -1007,14 +1007,14 @@
     <row r="1" ht="39.75" customHeight="1" s="42">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>BLAISE KINGKO, GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v15 ]</t>
+          <t>BLAISE KINGKO, GRC INTELLIGENCE &amp; RISK REGISTER   [ LIVE VERSION: v16 ]</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" s="42">
       <c r="A2" s="44" t="inlineStr">
         <is>
-          <t>LIVE VERSION: v15.  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-10-12   |   See 'Version Log' tab for history.</t>
+          <t>LIVE VERSION: v16.  This file is the current, authoritative register (continuously updated).   |   Sources: CISA KEV | US-CERT | NIST NVD | AWS/Azure Bulletins | AI Governance Updates | CISA/NSA/FBI Advisories | Supplementary news log   |   Frameworks: NIST CSF 2.0 | ISO 27001 | NIST 800-53 | CIS Controls | NIST AI RMF | ISO 42001 | EU AI Act   |   Last Updated: 2026-10-19   |   See 'Version Log' tab for history.</t>
         </is>
       </c>
     </row>
@@ -12908,7 +12908,7 @@
       </c>
       <c r="X105" s="53" t="inlineStr">
         <is>
-          <t>CVSS 9.3. Patch released concurrently with disclosure; exploitation nonetheless began within hours of public PoC release (190 attempts from 32 IPs in 10 countries within two days per Previdian telemetry). Not yet added to CISA KEV as of this report despite confirmed active exploitation; flagged for monitoring. Full case-study bundle published.</t>
+          <t>CVSS 9.3. Patch released concurrently with disclosure; exploitation nonetheless began within hours of public PoC release (190 attempts from 32 IPs in 10 countries within two days per Previdian telemetry). Not yet added to CISA KEV as of this report despite confirmed active exploitation; flagged for monitoring. Full case-study bundle published. UPDATE (2026-10-19): CISA added CVE-2026-21589 to the KEV catalog on 2026-10-15, confirming the active-exploitation status already reflected in this entry's Critical rating; no score change, logged per the duplicate-row-check rule rather than as a new row.</t>
         </is>
       </c>
     </row>
@@ -13143,6 +13143,942 @@
       <c r="X107" s="53" t="inlineStr">
         <is>
           <t>Non-CVE regulatory development, logged per this program's precedent of registering material EU AI Act timeline changes (cf. RR-004/RR-009 revision in v5, and the Article 50 enforcement-start entry in v8). No full bundle built; this is a confirmed regulatory development without an accompanying new technical finding. Folded into Executive Report AI Governance Watch and Compliance Posture narrative as well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" s="42">
+      <c r="A108" s="52" t="inlineStr">
+        <is>
+          <t>RR-104</t>
+        </is>
+      </c>
+      <c r="B108" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C108" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D108" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-104935</t>
+        </is>
+      </c>
+      <c r="E108" s="53" t="inlineStr">
+        <is>
+          <t>Ivanti Connect Secure authentication bypass by spoofing (CWE-290) allowing an unauthenticated remote attacker to execute arbitrary commands on the SSL VPN gateway; exploited as a zero-day against a limited set of customers before disclosure, chained by the attacker with a second, still-unpatched privilege-escalation flaw</t>
+        </is>
+      </c>
+      <c r="F108" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G108" s="53" t="inlineStr">
+        <is>
+          <t>VPN / Remote Access Gateway</t>
+        </is>
+      </c>
+      <c r="H108" s="53" t="inlineStr">
+        <is>
+          <t>Ivanti Connect Secure 25.1.1.1 and prior; 25.1.2.2 and prior; 22.8R2.4 and prior</t>
+        </is>
+      </c>
+      <c r="I108" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-02, DE.CM-01, RS.MI-02 | NIST 800-53: IA-2, SI-2, SC-7, IR-4 | ISO 27001: A.8.5, A.8.8 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J108" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification and Authentication</t>
+        </is>
+      </c>
+      <c r="K108" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L108" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M108" s="52">
+        <f>K108*L108</f>
+        <v/>
+      </c>
+      <c r="N108" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O108" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P108" s="53" t="inlineStr">
+        <is>
+          <t>Standard perimeter firewalling does not mitigate this flaw; the vulnerable logic is in the gateway's own authentication path, which is intentionally internet-facing</t>
+        </is>
+      </c>
+      <c r="Q108" s="52" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="R108" s="53" t="inlineStr">
+        <is>
+          <t>Apply vendor fix (25.1.1.2 / 25.1.3.0 or 25.1.3.1 / 22.8R2.5 per branch) immediately, outside the normal patch cycle; check against Volexity's published indicators for pre-disclosure compromise; track Ivanti's pending fix for the companion privilege-escalation flaw used in the observed attack chain</t>
+        </is>
+      </c>
+      <c r="S108" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T108" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U108" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V108" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W108" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X108" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 8.6. Exploited pre-disclosure against a limited customer set per Volexity; attack chain also used a second, still-unpatched privilege-escalation flaw Ivanti plans to fix separately, so patching this CVE alone does not guarantee an already-compromised appliance is clean. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" s="42">
+      <c r="A109" s="52" t="inlineStr">
+        <is>
+          <t>RR-105</t>
+        </is>
+      </c>
+      <c r="B109" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C109" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D109" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-76519</t>
+        </is>
+      </c>
+      <c r="E109" s="53" t="inlineStr">
+        <is>
+          <t>Relative path-traversal vulnerability (CWE-23) in Cisco Secure Email Gateway's File Reputation (AMP) attachment scanning, allowing an unauthenticated attacker to plant files and execute commands as root via a single crafted email attachment; no vendor-acknowledged workaround exists</t>
+        </is>
+      </c>
+      <c r="F109" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G109" s="53" t="inlineStr">
+        <is>
+          <t>Email Security Gateway</t>
+        </is>
+      </c>
+      <c r="H109" s="53" t="inlineStr">
+        <is>
+          <t>Cisco Secure Email Gateway (physical/virtual appliances, AsyncOS), File Reputation/AMP enabled, Content Scanner Tools below 25.3.0.5525</t>
+        </is>
+      </c>
+      <c r="I109" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-06, DE.CM-01, RS.MI-02 | NIST 800-53: SI-10, SI-2, SC-7, IR-4 | ISO 27001: A.8.8, A.8.26 | CIS Control 16</t>
+        </is>
+      </c>
+      <c r="J109" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K109" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L109" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M109" s="52">
+        <f>K109*L109</f>
+        <v/>
+      </c>
+      <c r="N109" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O109" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P109" s="53" t="inlineStr">
+        <is>
+          <t>None effective; the appliance's own attachment-scanning feature is the vulnerable component, and disabling it removes the malware-scanning protection it exists to provide</t>
+        </is>
+      </c>
+      <c r="Q109" s="52" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="R109" s="53" t="inlineStr">
+        <is>
+          <t>Update Content Scanner Tools to 25.3.0.5525 or later immediately (no reboot required); upgrade AsyncOS per branch (15.5.5-014 for 15.5, 16.5.0-780 for 16.5 and below; migrate any 16.0 appliance); run system-log check for prior compromise</t>
+        </is>
+      </c>
+      <c r="S109" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T109" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U109" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V109" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="W109" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X109" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 9.8. Cisco confirms active exploitation and states no workaround exists; Secure Email Cloud Gateway customers already protected, on-premises physical/virtual appliances are the exposed population. Full case-study bundle published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" s="42">
+      <c r="A110" s="52" t="inlineStr">
+        <is>
+          <t>RR-106</t>
+        </is>
+      </c>
+      <c r="B110" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C110" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D110" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-102764</t>
+        </is>
+      </c>
+      <c r="E110" s="53" t="inlineStr">
+        <is>
+          <t>Authentication-bypass vulnerability in BeyondTrust Remote Support exploited as a zero-day since late August 2026 by a suspected China-nexus espionage actor (Mandiant: Armory Castle/UNC5221; CrowdStrike: Warp Panda), who escalated to root, deployed the Sawfly web shell and Bareclaw tunneler malware, wiped logs, and moved laterally via stolen administrator credentials</t>
+        </is>
+      </c>
+      <c r="F110" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G110" s="53" t="inlineStr">
+        <is>
+          <t>Privileged Remote Access / IT Support Tooling</t>
+        </is>
+      </c>
+      <c r="H110" s="53" t="inlineStr">
+        <is>
+          <t>BeyondTrust Remote Support 26.2.3 and earlier (self-hosted); Privileged Remote Access patched as a precaution</t>
+        </is>
+      </c>
+      <c r="I110" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-02, DE.CM-01, RS.MI-02, RC.CO-01 | NIST 800-53: IA-2, AC-6, SI-2, IR-4, AU-6 | ISO 27001: A.8.5, A.5.24, A.8.15 | CIS Controls 5, 6, 8</t>
+        </is>
+      </c>
+      <c r="J110" s="53" t="inlineStr">
+        <is>
+          <t>IA — Identification and Authentication</t>
+        </is>
+      </c>
+      <c r="K110" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L110" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M110" s="52">
+        <f>K110*L110</f>
+        <v/>
+      </c>
+      <c r="N110" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O110" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P110" s="53" t="inlineStr">
+        <is>
+          <t>None; the authentication layer itself was the point of failure on a tool designed for trusted external remote access</t>
+        </is>
+      </c>
+      <c r="Q110" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R110" s="53" t="inlineStr">
+        <is>
+          <t>Patch every self-hosted instance immediately; engage an independent forensic review of all internet-reachable instances for Mandiant's published indicators (SUID escalation, Sawfly web shell, Bareclaw tunneler); rotate credentials used on affected appliances; implement centralized off-box audit logging</t>
+        </is>
+      </c>
+      <c r="S110" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 5.1 / 6.8 — Account and Access Control Management</t>
+        </is>
+      </c>
+      <c r="T110" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U110" s="52" t="inlineStr">
+        <is>
+          <t>Open — Emergency</t>
+        </is>
+      </c>
+      <c r="V110" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W110" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X110" s="53" t="inlineStr">
+        <is>
+          <t>Exploitation confirmed by Mandiant/GTIG to have begun in late August 2026, roughly seven weeks before CISA's 2026-10-16 KEV addition; over 1,400 internet-exposed instances identified by Shadowserver (patch status among them unconfirmed). Full case-study bundle published. CISA KEV due date not confirmed in sources reviewed for this entry; confirm against the primary CISA catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" s="42">
+      <c r="A111" s="52" t="inlineStr">
+        <is>
+          <t>RR-107</t>
+        </is>
+      </c>
+      <c r="B111" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C111" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D111" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-0322</t>
+        </is>
+      </c>
+      <c r="E111" s="53" t="inlineStr">
+        <is>
+          <t>Authenticated remote code execution vulnerability in the PAN-OS management interface allowing root-level command execution; Palo Alto Networks reports very limited exploitation tied to three identified source IPs</t>
+        </is>
+      </c>
+      <c r="F111" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G111" s="53" t="inlineStr">
+        <is>
+          <t>Network Perimeter Firewall</t>
+        </is>
+      </c>
+      <c r="H111" s="53" t="inlineStr">
+        <is>
+          <t>PAN-OS on PA-Series and VM-Series firewalls, and Panorama (virtual and M-Series); Cloud NGFW and Prisma Access unaffected</t>
+        </is>
+      </c>
+      <c r="I111" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, DE.CM-01 | NIST 800-53: AC-6, SI-2, SC-7 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J111" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K111" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="L111" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M111" s="52">
+        <f>K111*L111</f>
+        <v/>
+      </c>
+      <c r="N111" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O111" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P111" s="53" t="inlineStr">
+        <is>
+          <t>Restricting management-interface access to a trusted internal network or jump box, per vendor guidance, is the primary existing mitigation; where unrestricted, exposure is significant</t>
+        </is>
+      </c>
+      <c r="Q111" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R111" s="53" t="inlineStr">
+        <is>
+          <t>Apply the patched build for the deployed branch (12.2.4+; 12.1/11.2/11.1/10.2 h-patches per vendor table); restrict the PAN-OS management interface to a dedicated jump box or trusted internal network immediately as a compensating control</t>
+        </is>
+      </c>
+      <c r="S111" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T111" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U111" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V111" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="W111" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X111" s="53" t="inlineStr">
+        <is>
+          <t>CVSS 8.6. Palo Alto Networks reports exploitation as 'very limited,' tied to three identified source IPs, narrower than this week's broadly-exploited Ivanti/Cisco/BeyondTrust findings; requires authenticated access to the management interface. No full bundle built given the narrower exploitation scope and the access precondition, consistent with this program's narrow-footprint precedent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" s="42">
+      <c r="A112" s="52" t="inlineStr">
+        <is>
+          <t>RR-108</t>
+        </is>
+      </c>
+      <c r="B112" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C112" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV</t>
+        </is>
+      </c>
+      <c r="D112" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-96951</t>
+        </is>
+      </c>
+      <c r="E112" s="53" t="inlineStr">
+        <is>
+          <t>Windows Shell security feature bypass allowing an attacker to circumvent a Windows protection mechanism; added to CISA KEV the same week as October's Patch Tuesday, reported at a record volume of roughly 1,413 CVEs</t>
+        </is>
+      </c>
+      <c r="F112" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G112" s="53" t="inlineStr">
+        <is>
+          <t>Endpoint / Workstation Operating System</t>
+        </is>
+      </c>
+      <c r="H112" s="53" t="inlineStr">
+        <is>
+          <t>Microsoft Windows (Shell component)</t>
+        </is>
+      </c>
+      <c r="I112" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-02, DE.CM-01 | NIST 800-53: SI-2, CM-6 | CIS Control 7</t>
+        </is>
+      </c>
+      <c r="J112" s="53" t="inlineStr">
+        <is>
+          <t>SI — System Integrity</t>
+        </is>
+      </c>
+      <c r="K112" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L112" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M112" s="52">
+        <f>K112*L112</f>
+        <v/>
+      </c>
+      <c r="N112" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O112" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P112" s="53" t="inlineStr">
+        <is>
+          <t>Standard Windows Update cadence; the feature bypass itself does not grant code execution but can facilitate a subsequent attack stage</t>
+        </is>
+      </c>
+      <c r="Q112" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R112" s="53" t="inlineStr">
+        <is>
+          <t>Apply the October 2026 Patch Tuesday cumulative update addressing CVE-2026-96951 across all managed Windows endpoints per standard emergency patch SLA</t>
+        </is>
+      </c>
+      <c r="S112" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 7.4 — Vulnerability Remediation Process</t>
+        </is>
+      </c>
+      <c r="T112" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U112" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V112" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W112" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X112" s="53" t="inlineStr">
+        <is>
+          <t>Part of Microsoft's October 2026 Patch Tuesday release (reported record ~1,413 CVEs). Security-feature-bypass class finding; no full bundle built given the narrower direct-impact profile relative to this week's unauthenticated perimeter RCE findings, consistent with narrow-impact precedent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" s="42">
+      <c r="A113" s="52" t="inlineStr">
+        <is>
+          <t>RR-109</t>
+        </is>
+      </c>
+      <c r="B113" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C113" s="53" t="inlineStr">
+        <is>
+          <t>Vendor Advisory (Ahsay) / Security Researcher Reporting</t>
+        </is>
+      </c>
+      <c r="D113" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2026-105133 / CVE-2026-105134</t>
+        </is>
+      </c>
+      <c r="E113" s="53" t="inlineStr">
+        <is>
+          <t>Exploitation chain in the AhsayCBS backup management console (session-handling flaw chained to remote code execution) under active exploitation to deploy web shells and cryptocurrency-mining malware; Ahsay confirmed its first patch attempt failed to fully remediate the flaw</t>
+        </is>
+      </c>
+      <c r="F113" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G113" s="53" t="inlineStr">
+        <is>
+          <t>Backup / Data Recovery Infrastructure</t>
+        </is>
+      </c>
+      <c r="H113" s="53" t="inlineStr">
+        <is>
+          <t>Ahsay AhsayCBS backup management console</t>
+        </is>
+      </c>
+      <c r="I113" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.PS-02, DE.CM-01, RC.RP-01 | NIST 800-53: SI-2, CP-9, CP-10 | CIS Control 11</t>
+        </is>
+      </c>
+      <c r="J113" s="53" t="inlineStr">
+        <is>
+          <t>CP — Contingency Planning / Recovery Infrastructure</t>
+        </is>
+      </c>
+      <c r="K113" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="L113" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="M113" s="52">
+        <f>K113*L113</f>
+        <v/>
+      </c>
+      <c r="N113" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="O113" s="52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="P113" s="53" t="inlineStr">
+        <is>
+          <t>None effective; the vendor's first patch attempt is confirmed to have failed to close the exploitation path</t>
+        </is>
+      </c>
+      <c r="Q113" s="52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="R113" s="53" t="inlineStr">
+        <is>
+          <t>Monitor Ahsay for a working corrective patch and apply immediately on release; in the interim, isolate the AhsayCBS console from direct internet exposure and audit for web-shell/cryptominer indicators of compromise on any internet-reachable instance</t>
+        </is>
+      </c>
+      <c r="S113" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 11.3 — Protect Recovery Data</t>
+        </is>
+      </c>
+      <c r="T113" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U113" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V113" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W113" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X113" s="53" t="inlineStr">
+        <is>
+          <t>Backup/recovery infrastructure compromise carries elevated business-continuity significance (cf. this program's RR-095 Storm-3168 backup-sabotage entry). No full bundle built given AhsayCBS's narrower, managed-service-provider-focused install base relative to this week's broadly-deployed perimeter findings. Vendor's initial patch confirmed failed; monitor for a working fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" s="42">
+      <c r="A114" s="52" t="inlineStr">
+        <is>
+          <t>RR-110</t>
+        </is>
+      </c>
+      <c r="B114" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C114" s="53" t="inlineStr">
+        <is>
+          <t>CISA KEV / Vendor Advisory (Fortinet)</t>
+        </is>
+      </c>
+      <c r="D114" s="53" t="inlineStr">
+        <is>
+          <t>CVE-2025-61624</t>
+        </is>
+      </c>
+      <c r="E114" s="53" t="inlineStr">
+        <is>
+          <t>Path-traversal vulnerability (CWE-22) in the Fortinet CLI (FortiOS, FortiPAM, FortiProxy, FortiSwitchManager) allowing an authenticated, privileged administrator to write or delete arbitrary files via crafted CLI command arguments</t>
+        </is>
+      </c>
+      <c r="F114" s="52" t="inlineStr">
+        <is>
+          <t>IT-OT-Threats</t>
+        </is>
+      </c>
+      <c r="G114" s="53" t="inlineStr">
+        <is>
+          <t>Network Security Appliance (Firewall / Proxy / Switch Management)</t>
+        </is>
+      </c>
+      <c r="H114" s="53" t="inlineStr">
+        <is>
+          <t>FortiOS 6.4-7.6.4, FortiPAM 1.0-1.7.0, FortiProxy 7.0-7.6.4, FortiSwitchManager 7.0.0-7.2.7</t>
+        </is>
+      </c>
+      <c r="I114" s="53" t="inlineStr">
+        <is>
+          <t>NIST CSF 2.0: PR.AA-05, DE.CM-01 | NIST 800-53: AC-6, SI-2 | CIS Control 6</t>
+        </is>
+      </c>
+      <c r="J114" s="53" t="inlineStr">
+        <is>
+          <t>AC — Access Control</t>
+        </is>
+      </c>
+      <c r="K114" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="L114" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M114" s="52">
+        <f>K114*L114</f>
+        <v/>
+      </c>
+      <c r="N114" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O114" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P114" s="53" t="inlineStr">
+        <is>
+          <t>Requires an already-authenticated, privileged administrator account; standard admin-account hardening and MFA substantially reduce exploitability</t>
+        </is>
+      </c>
+      <c r="Q114" s="52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R114" s="53" t="inlineStr">
+        <is>
+          <t>Apply Fortinet's corrective release per advisory FG-IR-26-122 when confirmed available for the organization's deployed branch; enforce MFA and least-privilege on all administrative accounts for affected products in the interim</t>
+        </is>
+      </c>
+      <c r="S114" s="52" t="inlineStr">
+        <is>
+          <t>CIS Control 6.5 — Require MFA for Administrative Access</t>
+        </is>
+      </c>
+      <c r="T114" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U114" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only</t>
+        </is>
+      </c>
+      <c r="V114" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W114" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X114" s="53" t="inlineStr">
+        <is>
+          <t>CVSS reporting is inconsistent across sources reviewed (Fortinet advisory lists 5.4 Medium; NVD lists 6.5 Medium); this run's sources also disagreed on exact KEV status and due date, so the 2026-10-16 addition date is logged per the most specific secondary source found and flagged here for confirmation against the primary CISA catalog in the next run. Requires authenticated, privileged access; no full bundle built given the low-likelihood precondition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" s="42">
+      <c r="A115" s="52" t="inlineStr">
+        <is>
+          <t>RR-111</t>
+        </is>
+      </c>
+      <c r="B115" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C115" s="53" t="inlineStr">
+        <is>
+          <t>AI Governance Update</t>
+        </is>
+      </c>
+      <c r="D115" s="53" t="inlineStr">
+        <is>
+          <t>N/A — GSA Clause 552.239-7001 (RGO-2026-01)</t>
+        </is>
+      </c>
+      <c r="E115" s="53" t="inlineStr">
+        <is>
+          <t>GSA's final clause 552.239-7001, 'Basic Safeguarding of Data within Large Language Model Artificial Intelligence Systems,' takes effect, imposing data-use restrictions, 72-hour incident reporting, model-change notice, and closeout/deletion obligations on federal contracts involving LLM, generative-assistant, chatbot, or agentic AI products that touch government data</t>
+        </is>
+      </c>
+      <c r="F115" s="52" t="inlineStr">
+        <is>
+          <t>AI-Governance</t>
+        </is>
+      </c>
+      <c r="G115" s="53" t="inlineStr">
+        <is>
+          <t>AI Procurement / Federal Contract Compliance Program</t>
+        </is>
+      </c>
+      <c r="H115" s="53" t="inlineStr">
+        <is>
+          <t>Any LLM, generative AI assistant, chatbot, or agentic AI product sold under a GSA-governed federal contract where government data is submitted to or produced by the system</t>
+        </is>
+      </c>
+      <c r="I115" s="53" t="inlineStr">
+        <is>
+          <t>NIST AI RMF: GOVERN 1.1, MAP 1.1 | NIST CSF 2.0: GV.OC-01 | ISO 42001: Clause 4.1, 8.4</t>
+        </is>
+      </c>
+      <c r="J115" s="53" t="inlineStr">
+        <is>
+          <t>GV — Governance</t>
+        </is>
+      </c>
+      <c r="K115" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L115" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="M115" s="52">
+        <f>K115*L115</f>
+        <v/>
+      </c>
+      <c r="N115" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O115" s="52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P115" s="53" t="inlineStr">
+        <is>
+          <t>Organizations already tracking federal AI-procurement developments as part of standing AI-governance programs have advance notice; others may be contractually bound as of this effective date without a compliance program in place</t>
+        </is>
+      </c>
+      <c r="Q115" s="52" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="R115" s="53" t="inlineStr">
+        <is>
+          <t>Determine applicability (material LLM functionality and government data flowing to/from the system); map data flows across subcontractors; establish a 72-hour incident-reporting escalation path; update contract-review checklists to flag the clause's override of conflicting commercial terms</t>
+        </is>
+      </c>
+      <c r="S115" s="52" t="inlineStr">
+        <is>
+          <t>N/A — Regulatory/Compliance Governance Item (no direct CIS Controls mapping)</t>
+        </is>
+      </c>
+      <c r="T115" s="53" t="inlineStr">
+        <is>
+          <t>Blaise Kingko</t>
+        </is>
+      </c>
+      <c r="U115" s="52" t="inlineStr">
+        <is>
+          <t>Open — Register-Only (Governance)</t>
+        </is>
+      </c>
+      <c r="V115" s="52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W115" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="X115" s="53" t="inlineStr">
+        <is>
+          <t>Non-CVE regulatory development, logged per this program's precedent of registering material AI-governance/procurement developments (cf. EU AI Act Digital Omnibus entry RR-103 last run). First binding, immediately-effective federal procurement clause specifically governing LLM data handling this program has logged. No full bundle built; folded into Executive Report AI Governance Watch and Compliance Posture narrative instead.</t>
         </is>
       </c>
     </row>
@@ -21278,7 +22214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
@@ -21844,7 +22780,7 @@
       </c>
       <c r="C19" s="41" t="inlineStr">
         <is>
-          <t>LIVE</t>
+          <t>ARCHIVED</t>
         </is>
       </c>
       <c r="D19" s="41" t="inlineStr">
@@ -21863,6 +22799,41 @@
       <c r="G19" s="41" t="inlineStr">
         <is>
           <t>Added 4 new risks from the 2026-10-05 to 2026-10-12 sweep. Two full case-study bundles built: a four-CVE legacy-software batch (CVE-2015-3306 ProFTPD, CVE-2015-5477 ISC BIND, CVE-2021-3199 ONLYOFFICE Docs Server, CVE-2023-22894 Strapi) added to CISA KEV 2026-10-08 under a 3-day federal remediation deadline, tied to a joint international advisory (AA26-281A) attributing active exploitation to the Flax Typhoon intrusion set enabled by sanctioned Integrity Technology Group, with a concurrent FBI/DOJ domain-seizure action against the group's scanning and phishing infrastructure; and Atlassian Data Center's unauthenticated arbitrary file-access vulnerability (CVE-2026-21589, CVSS 9.3) across eight self-hosted products, patched at disclosure on 2026-10-05 but exploited within hours of public PoC release, with a documented escalation path to full Jira administrator takeover via Crowd-integrated deployments; not yet CISA KEV-listed as of this report despite confirmed active exploitation. Two register-only entries (no full bundle, per narrow-precondition/regulatory-development precedent): Amazon Bedrock AgentCore Starter Toolkit code-injection/SSRF pair (CVE-2026-105812, CVE-2026-106032), continuing this program's recurring AI-agent-platform trust-boundary finding category, scoped narrowly by the tool's deprecated status and import-action precondition; and the EU AI Act Digital Omnibus entering into force, deferring Annex III high-risk obligations to December 2027, the program's second documented compliance-easing data point in successive runs (after CMMC Phase 2's suspension). Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows found. Column-alignment spot check run and passed for all 4 new rows before save (G/H populated, K/L numeric 1-5, M=K*L formula verified, INHERENT RISK and NOTES populated for every row). FRAMEWORK UPDATE: FedRAMP 20x's CR26 change request went live 2026-10-06, replacing narrative assessment documentation with Key Security Indicators and machine-readable evidence for Classes A-C (Class D/High remains on Rev5 pending a 2027 pilot); Frameworks README updated to reflect this operational change to the existing FedRAMP entry. NIST Special Publication 1353 (draft, AI-assisted CSF 2.0 analysis and reporting) remains open for public comment through 2026-10-15; noted as a watch item in this week's Executive Report, not added to the Frameworks README while still in draft. A new US federal AI oversight structure (an interagency 'Super Intelligence Force' with a 120-day risk-report deliverable) was announced this window; reviewed and intentionally not logged as a register row, since it carries no defined technical or compliance obligation yet, consistent with this program's no-padding principle, folded into the Executive Report AI Governance Watch narrative instead. SUPPLEMENTARY CROSS-CHECK: the supplementary news log covering this report period was reviewed; none of its cybersecurity-adjacent mentions (legacy-CVE KEV batch, Atlassian flaw context, FedRAMP 20x, EU AI Act Omnibus, NIST SP 1353, Super Intelligence Force) were logged on the log's own word, each was independently verified against CISA, vendor, or primary regulatory sources before being reflected above or in this week's Executive Report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>v16</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>GRC_Intelligence_Risk_Register_2026-10-19.xlsx</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>RR-104 - RR-111 (new); RR-101 (updated, no new row)</t>
+        </is>
+      </c>
+      <c r="F20" s="41" t="n">
+        <v>115</v>
+      </c>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>Added 8 new risks from the 2026-10-12 to 2026-10-19 sweep. Three full case-study bundles built: Ivanti Connect Secure authentication-bypass-to-command-execution (CVE-2026-104935, CVSS 8.6, exploited pre-disclosure, chained with a still-unpatched privilege-escalation flaw); Cisco Secure Email Gateway path traversal to root command execution via a crafted email attachment (CVE-2026-76519, CVSS 9.8, confirmed active exploitation, no vendor workaround exists); and BeyondTrust Remote Support authentication bypass exploited for roughly seven weeks by a suspected China-nexus espionage actor (CVE-2026-102764, Mandiant: Armory Castle/UNC5221; CrowdStrike: Warp Panda), with root-level compromise, web-shell/tunneler malware, log wiping, and lateral movement via stolen credentials, over 1,400 internet-exposed instances identified by Shadowserver. Four register-only entries (no full bundle, per narrow-footprint/precondition precedent): PAN-OS management-interface authenticated RCE (CVE-2026-0322, CVSS 8.6, Palo Alto Networks reports exploitation as 'very limited,' tied to three source IPs); Windows Shell security-feature bypass (CVE-2026-96951) logged within October's record ~1,413-CVE Patch Tuesday; an AhsayCBS backup-console exploitation chain (CVE-2026-105133/105134) used to deploy web shells and cryptominers, notable because Ahsay's first patch attempt confirmed failed; and a Fortinet CLI path-traversal flaw (CVE-2025-61624) requiring authenticated privileged access, logged with an explicit data-quality caveat given inconsistent CVSS and KEV-status reporting across sources. One non-CVE AI-governance entry: GSA's final clause 552.239-7001 on LLM data safeguarding in federal contracts took effect 2026-10-19, the first binding, immediately-effective federal procurement clause of its kind this program has logged; folded into the Executive Report AI Governance Watch and Compliance Posture narrative, no full bundle built, consistent with this program's regulatory-development precedent (cf. RR-103 last run). UPDATE TO EXISTING ENTRY: RR-101 (Atlassian CVE-2026-21589) was officially added to the CISA KEV catalog on 2026-10-15, confirming its existing Critical rating; no score change, so per the duplicate-row-check rule this was logged as a Notes-field update to the existing row rather than a new row. SUPPLEMENTARY CROSS-CHECK: the supplementary news log covering this report period (2026-10-12 through 2026-10-16 entries, the most recent available) was reviewed for cybersecurity-adjacent mentions not already captured by the primary sweep; all items it referenced (Ivanti Connect Secure, the October Patch Tuesday batch, Atlassian KEV status, GSA 552.239-7001, FedRAMP FY26 scorecard, EU AI Act Omnibus dates) were independently verified against CISA, vendor, or primary regulatory sources before being reflected above or in this week's Executive Report; none were logged on the log's own word alone. No prior-week coverage gaps were surfaced during this cross-check. Dedup check performed against all CVE/Advisory IDs on file; no duplicate rows created (RR-101 updated in place per above). Column-alignment spot check run and passed for all 8 new rows before save (G/H populated for every row, K/L numeric 1-5, M=K*L formula verified, INHERENT RISK and NOTES populated for every row). No new frameworks used this run; Frameworks README reviewed, no update needed.</t>
         </is>
       </c>
     </row>

</xml_diff>